<commit_message>
Atualização automática: pagamentos (14/09/2026 13:57)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/01_Bases_Originais/005_CELOG_2025/005_CELOG-PAMALS_2025 online.xlsx
+++ b/Contrato 005/Dashboard/01_Bases_Originais/005_CELOG_2025/005_CELOG-PAMALS_2025 online.xlsx
@@ -36,12 +36,12 @@
     <t>2025NE000005</t>
   </si>
   <si>
+    <t>C25375</t>
+  </si>
+  <si>
     <t>Controle de pagamentos</t>
   </si>
   <si>
-    <t>C25375</t>
-  </si>
-  <si>
     <t>Ordenador de Despesas</t>
   </si>
   <si>
@@ -66,6 +66,12 @@
     <t>25E0387</t>
   </si>
   <si>
+    <t>2025NE000371</t>
+  </si>
+  <si>
+    <t>25E0389</t>
+  </si>
+  <si>
     <t>Número Contrato</t>
   </si>
   <si>
@@ -84,12 +90,21 @@
     <t>Prazo Final de Vigência</t>
   </si>
   <si>
+    <t>2025NE000413</t>
+  </si>
+  <si>
     <t>Status</t>
   </si>
   <si>
+    <t>C25501</t>
+  </si>
+  <si>
     <t>Ação</t>
   </si>
   <si>
+    <t>25E0403</t>
+  </si>
+  <si>
     <t>PAG</t>
   </si>
   <si>
@@ -105,15 +120,12 @@
     <t>Valor Empenhado</t>
   </si>
   <si>
-    <t>2025NE000371</t>
+    <t>20SP</t>
   </si>
   <si>
     <t>Valor Liquidado</t>
   </si>
   <si>
-    <t>25E0389</t>
-  </si>
-  <si>
     <t>Saldo (Valor a Faturar)</t>
   </si>
   <si>
@@ -129,39 +141,30 @@
     <t>Editar</t>
   </si>
   <si>
-    <t>2025NE000413</t>
-  </si>
-  <si>
-    <t>C25501</t>
-  </si>
-  <si>
-    <t>25E0403</t>
+    <t>2025NE000414</t>
+  </si>
+  <si>
+    <t>C25525</t>
+  </si>
+  <si>
+    <t>25E0431</t>
   </si>
   <si>
     <t>005/CELOG-PAMALS/2025</t>
   </si>
   <si>
+    <t>21EM</t>
+  </si>
+  <si>
     <t>CELOG</t>
   </si>
   <si>
     <t>PAMALS</t>
   </si>
   <si>
-    <t>20SP</t>
-  </si>
-  <si>
-    <t>2025NE000414</t>
-  </si>
-  <si>
-    <t>C25525</t>
-  </si>
-  <si>
     <t>Vigente</t>
   </si>
   <si>
-    <t>25E0431</t>
-  </si>
-  <si>
     <t>2048 20YJ 21EM 219C 20SP 20X7 2000</t>
   </si>
   <si>
@@ -171,9 +174,6 @@
     <t>R$</t>
   </si>
   <si>
-    <t>21EM</t>
-  </si>
-  <si>
     <t>VEE ONE-MANUTENCAO E SERVICOS TECNICOS LTDA</t>
   </si>
   <si>
@@ -195,27 +195,39 @@
     <t>25E0731</t>
   </si>
   <si>
+    <t>2025NE000774</t>
+  </si>
+  <si>
+    <t>25E0737</t>
+  </si>
+  <si>
     <t>Módulo</t>
   </si>
   <si>
     <t>Referência</t>
   </si>
   <si>
-    <t>2025NE000774</t>
-  </si>
-  <si>
-    <t>25E0737</t>
+    <t>2025NE000843</t>
+  </si>
+  <si>
+    <t>C25630</t>
   </si>
   <si>
     <t>Nº recibo</t>
   </si>
   <si>
+    <t>25E0787</t>
+  </si>
+  <si>
     <t>Nº</t>
   </si>
   <si>
     <t>Data</t>
   </si>
   <si>
+    <t>219C</t>
+  </si>
+  <si>
     <t>Empenho</t>
   </si>
   <si>
@@ -231,30 +243,18 @@
     <t>Ordem de Pagamento</t>
   </si>
   <si>
+    <t>2025NE001065</t>
+  </si>
+  <si>
+    <t>25E0999</t>
+  </si>
+  <si>
     <t>Faturado</t>
   </si>
   <si>
     <t>Pendente</t>
   </si>
   <si>
-    <t>2025NE000843</t>
-  </si>
-  <si>
-    <t>C25630</t>
-  </si>
-  <si>
-    <t>25E0787</t>
-  </si>
-  <si>
-    <t>219C</t>
-  </si>
-  <si>
-    <t>2025NE001065</t>
-  </si>
-  <si>
-    <t>25E0999</t>
-  </si>
-  <si>
     <t>2025NE001200</t>
   </si>
   <si>
@@ -282,15 +282,15 @@
     <t xml:space="preserve">2025NE000369 </t>
   </si>
   <si>
+    <t>2025NE001627</t>
+  </si>
+  <si>
+    <t>25E1475</t>
+  </si>
+  <si>
     <t>2025NP001980</t>
   </si>
   <si>
-    <t>2025NE001627</t>
-  </si>
-  <si>
-    <t>25E1475</t>
-  </si>
-  <si>
     <t>2025NE001629</t>
   </si>
   <si>
@@ -318,12 +318,21 @@
     <t>25E1537</t>
   </si>
   <si>
+    <t>MAR/25</t>
+  </si>
+  <si>
     <t>2025NE001690</t>
   </si>
   <si>
     <t>25E1538</t>
   </si>
   <si>
+    <t>2025NE000367, 2025NE000369, 2025NE000371, 2025NE000413</t>
+  </si>
+  <si>
+    <t>2025NP001979</t>
+  </si>
+  <si>
     <t>2025NE001823</t>
   </si>
   <si>
@@ -333,25 +342,28 @@
     <t>25E1666</t>
   </si>
   <si>
-    <t>MAR/25</t>
+    <t>ABR/25</t>
+  </si>
+  <si>
+    <t>2025NE000413, 2025NE000414, 2025NE000559</t>
   </si>
   <si>
     <t>2025NE001828</t>
   </si>
   <si>
+    <t>2025NP002341</t>
+  </si>
+  <si>
     <t>C25869</t>
   </si>
   <si>
     <t>25E1667</t>
   </si>
   <si>
-    <t>2025NE000367, 2025NE000369, 2025NE000371, 2025NE000413</t>
-  </si>
-  <si>
     <t>20YJ</t>
   </si>
   <si>
-    <t>2025NP001979</t>
+    <t>MAI/25</t>
   </si>
   <si>
     <t>2025NE001830</t>
@@ -369,19 +381,16 @@
     <t>25E2021</t>
   </si>
   <si>
-    <t>ABR/25</t>
+    <t>2025NP002884</t>
   </si>
   <si>
     <t>2025NE002237</t>
   </si>
   <si>
-    <t>2025NE000413, 2025NE000414, 2025NE000559</t>
-  </si>
-  <si>
     <t>25E2058</t>
   </si>
   <si>
-    <t>2025NP002341</t>
+    <t>JUN/25</t>
   </si>
   <si>
     <t>2026NE000330</t>
@@ -391,51 +400,6 @@
   </si>
   <si>
     <t>26E0320</t>
-  </si>
-  <si>
-    <t>MAI/25</t>
-  </si>
-  <si>
-    <t>2026NE000388</t>
-  </si>
-  <si>
-    <t>C26193</t>
-  </si>
-  <si>
-    <t>26E0375</t>
-  </si>
-  <si>
-    <t>2025NP002884</t>
-  </si>
-  <si>
-    <t>2026NE000748</t>
-  </si>
-  <si>
-    <t>C26312</t>
-  </si>
-  <si>
-    <t>26E0709</t>
-  </si>
-  <si>
-    <t>2026NE000816</t>
-  </si>
-  <si>
-    <t>C26324</t>
-  </si>
-  <si>
-    <t>26E0776</t>
-  </si>
-  <si>
-    <t>JUN/25</t>
-  </si>
-  <si>
-    <t>2026NE000817</t>
-  </si>
-  <si>
-    <t>C26326</t>
-  </si>
-  <si>
-    <t>26E0777</t>
   </si>
   <si>
     <t>2025NE000005,
@@ -447,52 +411,55 @@
     <t>2025NP400522</t>
   </si>
   <si>
-    <t>2026NE000842</t>
-  </si>
-  <si>
-    <t>26E0803</t>
+    <t>2026NE000388</t>
   </si>
   <si>
     <t>JUL/25</t>
   </si>
   <si>
-    <t>2026NE000944</t>
+    <t>C26193</t>
+  </si>
+  <si>
+    <t>26E0375</t>
   </si>
   <si>
     <t>2025NE000843, 2025NE001200</t>
   </si>
   <si>
-    <t>26E0906</t>
-  </si>
-  <si>
     <t>2025NP003724</t>
   </si>
   <si>
     <t>AGO/25</t>
   </si>
   <si>
-    <t>2026NE001015</t>
-  </si>
-  <si>
-    <t>C26363</t>
-  </si>
-  <si>
-    <t>26E0959</t>
+    <t>2026NE000748</t>
+  </si>
+  <si>
+    <t>C26312</t>
+  </si>
+  <si>
+    <t>26E0709</t>
   </si>
   <si>
     <t>2025NP004558</t>
   </si>
   <si>
-    <t>20XV</t>
-  </si>
-  <si>
     <t>SET/25</t>
+  </si>
+  <si>
+    <t>2026NE000816</t>
   </si>
   <si>
     <t>2025NE001688 
 2025NE001828</t>
   </si>
   <si>
+    <t>C26324</t>
+  </si>
+  <si>
+    <t>26E0776</t>
+  </si>
+  <si>
     <t>2025NP004897</t>
   </si>
   <si>
@@ -505,28 +472,61 @@
     <t>2025NP004932</t>
   </si>
   <si>
+    <t>2026NE000817</t>
+  </si>
+  <si>
+    <t>C26326</t>
+  </si>
+  <si>
+    <t>26E0777</t>
+  </si>
+  <si>
     <t>NOV/25</t>
   </si>
   <si>
+    <t>2026NE000842</t>
+  </si>
+  <si>
     <t>2025NE001687, 2025NE001689, 2025NE001690, 2025NE001823, 2025NE001830, 2025NE002237</t>
   </si>
   <si>
+    <t>26E0803</t>
+  </si>
+  <si>
     <t>2026NP400440</t>
   </si>
   <si>
+    <t>2026NE000944</t>
+  </si>
+  <si>
     <t>DEZ/25</t>
   </si>
   <si>
+    <t>26E0906</t>
+  </si>
+  <si>
     <t>2025NE001065, 2025NE002200</t>
   </si>
   <si>
     <t>2026NP400412</t>
   </si>
   <si>
+    <t>2026NE001015</t>
+  </si>
+  <si>
+    <t>C26363</t>
+  </si>
+  <si>
     <t>JAN/26</t>
   </si>
   <si>
+    <t>26E0959</t>
+  </si>
+  <si>
     <t>2026NP401035</t>
+  </si>
+  <si>
+    <t>20XV</t>
   </si>
   <si>
     <t>FEV/26</t>
@@ -894,33 +894,33 @@
     <xf borderId="0" fillId="0" fontId="2" numFmtId="164" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
       <alignment readingOrder="0"/>
     </xf>
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0"/>
+    </xf>
     <xf borderId="0" fillId="4" fontId="2" numFmtId="0" xfId="0" applyFill="1" applyFont="1"/>
     <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0"/>
+      <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="0" fillId="2" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" vertical="center"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="11" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
+      <alignment horizontal="center" readingOrder="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="164" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="0" fillId="5" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" vertical="center"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="11" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="4" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="0" fillId="4" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
       <alignment vertical="center"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="164" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
-      <alignment horizontal="center" readingOrder="0"/>
-    </xf>
     <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment vertical="center"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="4" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
-      <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
@@ -941,11 +941,11 @@
     <xf borderId="0" fillId="6" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
       <alignment horizontal="right" readingOrder="0"/>
     </xf>
+    <xf borderId="1" fillId="0" fontId="5" numFmtId="165" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf borderId="0" fillId="0" fontId="2" numFmtId="4" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="right" readingOrder="0"/>
-    </xf>
-    <xf borderId="1" fillId="0" fontId="5" numFmtId="165" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
-      <alignment vertical="center"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment shrinkToFit="0" wrapText="1"/>
@@ -999,12 +999,12 @@
     <xf borderId="1" fillId="8" fontId="7" numFmtId="168" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="169" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
-      <alignment horizontal="center" readingOrder="0"/>
-    </xf>
     <xf borderId="3" fillId="0" fontId="10" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
     <xf borderId="1" fillId="8" fontId="9" numFmtId="168" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="169" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
+      <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="1" fillId="0" fontId="8" numFmtId="166" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
@@ -1437,22 +1437,22 @@
       <c r="S1" s="1"/>
       <c r="T1" s="1"/>
       <c r="U1" s="1"/>
-      <c r="V1" s="4"/>
+      <c r="V1" s="5"/>
     </row>
     <row r="2" ht="59.25" customHeight="1">
-      <c r="A2" s="6"/>
-      <c r="B2" s="8" t="s">
-        <v>2</v>
-      </c>
-      <c r="V2" s="10"/>
-      <c r="W2" s="12"/>
-      <c r="X2" s="12"/>
-      <c r="Y2" s="12"/>
-      <c r="Z2" s="12"/>
-      <c r="AA2" s="12"/>
-      <c r="AB2" s="12"/>
-      <c r="AC2" s="12"/>
-      <c r="AD2" s="12"/>
+      <c r="A2" s="7"/>
+      <c r="B2" s="10" t="s">
+        <v>3</v>
+      </c>
+      <c r="V2" s="12"/>
+      <c r="W2" s="13"/>
+      <c r="X2" s="13"/>
+      <c r="Y2" s="13"/>
+      <c r="Z2" s="13"/>
+      <c r="AA2" s="13"/>
+      <c r="AB2" s="13"/>
+      <c r="AC2" s="13"/>
+      <c r="AD2" s="13"/>
     </row>
     <row r="3" ht="12.75" customHeight="1">
       <c r="A3" s="1"/>
@@ -1476,85 +1476,85 @@
       <c r="S3" s="14"/>
       <c r="T3" s="14"/>
       <c r="U3" s="14"/>
-      <c r="V3" s="4"/>
+      <c r="V3" s="5"/>
     </row>
     <row r="4" ht="12.75" customHeight="1">
       <c r="A4" s="15"/>
       <c r="B4" s="15"/>
       <c r="C4" s="16" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="D4" s="16" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="E4" s="16" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="F4" s="16" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="G4" s="17" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="H4" s="17" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="I4" s="16" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="J4" s="16" t="s">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="K4" s="16" t="s">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="L4" s="16" t="s">
-        <v>21</v>
+        <v>26</v>
       </c>
       <c r="M4" s="17" t="s">
-        <v>22</v>
+        <v>27</v>
       </c>
       <c r="N4" s="17" t="s">
-        <v>23</v>
+        <v>28</v>
       </c>
       <c r="O4" s="17" t="s">
-        <v>24</v>
+        <v>29</v>
       </c>
       <c r="P4" s="17" t="s">
-        <v>26</v>
+        <v>31</v>
       </c>
       <c r="Q4" s="17" t="s">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="R4" s="16" t="s">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="S4" s="16" t="s">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="T4" s="16" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="U4" s="16" t="s">
-        <v>32</v>
-      </c>
-      <c r="V4" s="4"/>
+        <v>36</v>
+      </c>
+      <c r="V4" s="5"/>
     </row>
     <row r="5" ht="12.75" customHeight="1">
       <c r="A5" s="15"/>
       <c r="B5" s="15"/>
       <c r="C5" s="18"/>
       <c r="D5" s="19" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="E5" s="19" t="s">
-        <v>37</v>
+        <v>42</v>
       </c>
       <c r="F5" s="19" t="s">
-        <v>38</v>
+        <v>43</v>
       </c>
       <c r="G5" s="19" t="s">
-        <v>38</v>
+        <v>43</v>
       </c>
       <c r="H5" s="20">
         <v>1564.0</v>
@@ -1563,42 +1563,42 @@
         <v>1564.0</v>
       </c>
       <c r="J5" s="19" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="K5" s="19" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="L5" s="19" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="M5" s="19" t="s">
-        <v>46</v>
-      </c>
-      <c r="N5" s="21">
+        <v>47</v>
+      </c>
+      <c r="N5" s="22">
         <v>9.165159737E7</v>
       </c>
-      <c r="O5" s="21">
+      <c r="O5" s="22">
         <v>7.254367932E7</v>
       </c>
-      <c r="P5" s="21">
+      <c r="P5" s="22">
         <v>1.910791805E7</v>
       </c>
-      <c r="Q5" s="21">
+      <c r="Q5" s="22">
         <v>8248487.61</v>
       </c>
-      <c r="R5" s="21">
+      <c r="R5" s="22">
         <v>1.085943044E7</v>
       </c>
       <c r="S5" s="19" t="s">
         <v>48</v>
       </c>
-      <c r="V5" s="4"/>
+      <c r="V5" s="5"/>
     </row>
     <row r="6" ht="12.75" customHeight="1">
       <c r="A6" s="15"/>
       <c r="B6" s="15"/>
       <c r="L6" s="23"/>
-      <c r="V6" s="4"/>
+      <c r="V6" s="5"/>
     </row>
     <row r="7" ht="12.75" customHeight="1">
       <c r="A7" s="24"/>
@@ -1617,50 +1617,50 @@
       <c r="N7" s="26"/>
       <c r="O7" s="26"/>
       <c r="P7" s="28"/>
-      <c r="V7" s="4"/>
+      <c r="V7" s="5"/>
     </row>
     <row r="8" ht="12.75" customHeight="1">
       <c r="A8" s="24"/>
       <c r="B8" s="24"/>
       <c r="C8" s="29" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="D8" s="29" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="E8" s="30" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="F8" s="29" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="G8" s="29" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="H8" s="29" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="I8" s="30" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="J8" s="29" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="K8" s="29" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="L8" s="31" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="M8" s="30" t="s">
-        <v>67</v>
+        <v>73</v>
       </c>
       <c r="N8" s="29" t="s">
-        <v>68</v>
+        <v>74</v>
       </c>
       <c r="O8" s="29"/>
       <c r="P8" s="28"/>
-      <c r="V8" s="4"/>
+      <c r="V8" s="5"/>
     </row>
     <row r="9" ht="19.5" customHeight="1">
       <c r="A9" s="24"/>
@@ -1691,7 +1691,7 @@
         <v>748504.24</v>
       </c>
       <c r="L9" s="36" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="M9" s="39">
         <f t="shared" ref="M9:M10" si="1">K9</f>
@@ -1700,14 +1700,14 @@
       <c r="N9" s="40"/>
       <c r="O9" s="26"/>
       <c r="P9" s="28"/>
-      <c r="V9" s="4"/>
+      <c r="V9" s="5"/>
     </row>
     <row r="10" ht="51.0" customHeight="1">
       <c r="A10" s="24"/>
       <c r="B10" s="24"/>
-      <c r="C10" s="42"/>
+      <c r="C10" s="41"/>
       <c r="D10" s="34" t="s">
-        <v>101</v>
+        <v>96</v>
       </c>
       <c r="E10" s="35" t="s">
         <v>81</v>
@@ -1719,7 +1719,7 @@
         <v>45775.0</v>
       </c>
       <c r="H10" s="36" t="s">
-        <v>105</v>
+        <v>99</v>
       </c>
       <c r="I10" s="37"/>
       <c r="J10" s="37">
@@ -1729,23 +1729,23 @@
         <v>1110378.24</v>
       </c>
       <c r="L10" s="36" t="s">
-        <v>107</v>
+        <v>100</v>
       </c>
       <c r="M10" s="39">
         <f t="shared" si="1"/>
         <v>1110378.24</v>
       </c>
-      <c r="N10" s="43"/>
+      <c r="N10" s="42"/>
       <c r="O10" s="26"/>
       <c r="P10" s="28"/>
-      <c r="V10" s="4"/>
+      <c r="V10" s="5"/>
     </row>
     <row r="11" ht="12.75" customHeight="1">
       <c r="A11" s="24"/>
       <c r="B11" s="24"/>
-      <c r="C11" s="42"/>
+      <c r="C11" s="41"/>
       <c r="D11" s="34" t="s">
-        <v>113</v>
+        <v>104</v>
       </c>
       <c r="E11" s="35" t="s">
         <v>81</v>
@@ -1757,7 +1757,7 @@
         <v>45799.0</v>
       </c>
       <c r="H11" s="36" t="s">
-        <v>115</v>
+        <v>105</v>
       </c>
       <c r="I11" s="37"/>
       <c r="J11" s="37">
@@ -1767,22 +1767,22 @@
         <v>974557.12</v>
       </c>
       <c r="L11" s="35" t="s">
-        <v>117</v>
+        <v>107</v>
       </c>
       <c r="M11" s="39">
         <v>974557.12</v>
       </c>
-      <c r="N11" s="43"/>
+      <c r="N11" s="42"/>
       <c r="O11" s="26"/>
       <c r="P11" s="28"/>
-      <c r="V11" s="4"/>
+      <c r="V11" s="5"/>
     </row>
     <row r="12" ht="27.75" customHeight="1">
       <c r="A12" s="24"/>
       <c r="B12" s="24"/>
-      <c r="C12" s="42"/>
+      <c r="C12" s="41"/>
       <c r="D12" s="34" t="s">
-        <v>121</v>
+        <v>111</v>
       </c>
       <c r="E12" s="35" t="s">
         <v>81</v>
@@ -1794,7 +1794,7 @@
         <v>45856.0</v>
       </c>
       <c r="H12" s="45" t="s">
-        <v>69</v>
+        <v>59</v>
       </c>
       <c r="I12" s="37"/>
       <c r="J12" s="37">
@@ -1804,7 +1804,7 @@
         <v>1402001.34</v>
       </c>
       <c r="L12" s="47" t="s">
-        <v>125</v>
+        <v>117</v>
       </c>
       <c r="M12" s="39">
         <v>1402001.34</v>
@@ -1812,14 +1812,14 @@
       <c r="N12" s="48"/>
       <c r="O12" s="26"/>
       <c r="P12" s="28"/>
-      <c r="V12" s="4"/>
+      <c r="V12" s="5"/>
     </row>
     <row r="13">
       <c r="A13" s="24"/>
       <c r="B13" s="24"/>
-      <c r="C13" s="42"/>
+      <c r="C13" s="41"/>
       <c r="D13" s="49" t="s">
-        <v>132</v>
+        <v>120</v>
       </c>
       <c r="E13" s="35" t="s">
         <v>81</v>
@@ -1831,7 +1831,7 @@
         <v>45856.0</v>
       </c>
       <c r="H13" s="36" t="s">
-        <v>136</v>
+        <v>124</v>
       </c>
       <c r="I13" s="44"/>
       <c r="J13" s="44">
@@ -1841,7 +1841,7 @@
         <v>1223702.3</v>
       </c>
       <c r="L13" s="35" t="s">
-        <v>137</v>
+        <v>125</v>
       </c>
       <c r="M13" s="39">
         <v>1223702.3</v>
@@ -1849,14 +1849,14 @@
       <c r="N13" s="48"/>
       <c r="O13" s="26"/>
       <c r="P13" s="50"/>
-      <c r="V13" s="4"/>
+      <c r="V13" s="5"/>
     </row>
     <row r="14">
       <c r="A14" s="24"/>
       <c r="B14" s="24"/>
-      <c r="C14" s="42"/>
+      <c r="C14" s="41"/>
       <c r="D14" s="49" t="s">
-        <v>140</v>
+        <v>127</v>
       </c>
       <c r="E14" s="35" t="s">
         <v>81</v>
@@ -1868,7 +1868,7 @@
         <v>45901.0</v>
       </c>
       <c r="H14" s="35" t="s">
-        <v>142</v>
+        <v>130</v>
       </c>
       <c r="I14" s="44"/>
       <c r="J14" s="44">
@@ -1878,22 +1878,22 @@
         <v>1011677.95</v>
       </c>
       <c r="L14" s="35" t="s">
-        <v>144</v>
+        <v>131</v>
       </c>
       <c r="M14" s="39">
         <v>1011677.95</v>
       </c>
-      <c r="N14" s="43"/>
+      <c r="N14" s="42"/>
       <c r="O14" s="26"/>
       <c r="P14" s="28"/>
-      <c r="V14" s="4"/>
+      <c r="V14" s="5"/>
     </row>
     <row r="15">
       <c r="A15" s="24"/>
       <c r="B15" s="24"/>
-      <c r="C15" s="42"/>
+      <c r="C15" s="41"/>
       <c r="D15" s="49" t="s">
-        <v>145</v>
+        <v>132</v>
       </c>
       <c r="E15" s="35" t="s">
         <v>81</v>
@@ -1915,21 +1915,21 @@
         <v>896744.06</v>
       </c>
       <c r="L15" s="35" t="s">
-        <v>149</v>
+        <v>136</v>
       </c>
       <c r="M15" s="39">
         <v>896744.06</v>
       </c>
       <c r="N15" s="48"/>
       <c r="O15" s="26"/>
-      <c r="V15" s="4"/>
+      <c r="V15" s="5"/>
     </row>
     <row r="16">
       <c r="A16" s="24"/>
       <c r="B16" s="24"/>
-      <c r="C16" s="42"/>
+      <c r="C16" s="41"/>
       <c r="D16" s="49" t="s">
-        <v>151</v>
+        <v>137</v>
       </c>
       <c r="E16" s="35" t="s">
         <v>81</v>
@@ -1941,7 +1941,7 @@
         <v>45957.0</v>
       </c>
       <c r="H16" s="35" t="s">
-        <v>152</v>
+        <v>139</v>
       </c>
       <c r="I16" s="44"/>
       <c r="J16" s="44">
@@ -1951,21 +1951,21 @@
         <v>919329.06</v>
       </c>
       <c r="L16" s="35" t="s">
-        <v>153</v>
+        <v>142</v>
       </c>
       <c r="M16" s="39">
         <v>919329.06</v>
       </c>
-      <c r="N16" s="43"/>
+      <c r="N16" s="42"/>
       <c r="O16" s="26"/>
-      <c r="V16" s="4"/>
+      <c r="V16" s="5"/>
     </row>
     <row r="17">
       <c r="A17" s="24"/>
       <c r="B17" s="24"/>
-      <c r="C17" s="42"/>
+      <c r="C17" s="41"/>
       <c r="D17" s="49" t="s">
-        <v>154</v>
+        <v>143</v>
       </c>
       <c r="E17" s="35"/>
       <c r="F17" s="35">
@@ -1975,7 +1975,7 @@
         <v>45972.0</v>
       </c>
       <c r="H17" s="35" t="s">
-        <v>155</v>
+        <v>144</v>
       </c>
       <c r="I17" s="35"/>
       <c r="J17" s="44">
@@ -1985,21 +1985,21 @@
         <v>1157009.26</v>
       </c>
       <c r="L17" s="35" t="s">
-        <v>156</v>
+        <v>145</v>
       </c>
       <c r="M17" s="39">
         <v>1157009.26</v>
       </c>
       <c r="N17" s="51"/>
       <c r="O17" s="26"/>
-      <c r="V17" s="4"/>
+      <c r="V17" s="5"/>
     </row>
     <row r="18">
       <c r="A18" s="24"/>
       <c r="B18" s="24"/>
-      <c r="C18" s="42"/>
+      <c r="C18" s="41"/>
       <c r="D18" s="49" t="s">
-        <v>157</v>
+        <v>149</v>
       </c>
       <c r="E18" s="35" t="s">
         <v>81</v>
@@ -2011,7 +2011,7 @@
         <v>46008.0</v>
       </c>
       <c r="H18" s="35" t="s">
-        <v>158</v>
+        <v>151</v>
       </c>
       <c r="I18" s="35"/>
       <c r="J18" s="44">
@@ -2021,7 +2021,7 @@
         <v>1214597.952</v>
       </c>
       <c r="L18" s="35" t="s">
-        <v>159</v>
+        <v>153</v>
       </c>
       <c r="M18" s="39">
         <v>1214597.952</v>
@@ -2037,9 +2037,9 @@
     <row r="19">
       <c r="A19" s="24"/>
       <c r="B19" s="24"/>
-      <c r="C19" s="42"/>
+      <c r="C19" s="41"/>
       <c r="D19" s="49" t="s">
-        <v>160</v>
+        <v>155</v>
       </c>
       <c r="E19" s="35" t="s">
         <v>81</v>
@@ -2051,7 +2051,7 @@
         <v>46042.0</v>
       </c>
       <c r="H19" s="35" t="s">
-        <v>161</v>
+        <v>157</v>
       </c>
       <c r="I19" s="44"/>
       <c r="J19" s="44">
@@ -2061,7 +2061,7 @@
         <v>967082.09</v>
       </c>
       <c r="L19" s="35" t="s">
-        <v>162</v>
+        <v>158</v>
       </c>
       <c r="M19" s="39">
         <v>967082.09</v>
@@ -2077,9 +2077,9 @@
     <row r="20">
       <c r="A20" s="24"/>
       <c r="B20" s="24"/>
-      <c r="C20" s="42"/>
+      <c r="C20" s="41"/>
       <c r="D20" s="49" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="E20" s="35"/>
       <c r="F20" s="35">
@@ -2089,7 +2089,7 @@
         <v>46078.0</v>
       </c>
       <c r="H20" s="35" t="s">
-        <v>98</v>
+        <v>101</v>
       </c>
       <c r="I20" s="44"/>
       <c r="J20" s="44">
@@ -2099,7 +2099,7 @@
         <v>719561.08</v>
       </c>
       <c r="L20" s="35" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="M20" s="39">
         <v>719561.08</v>
@@ -2115,7 +2115,7 @@
     <row r="21">
       <c r="A21" s="24"/>
       <c r="B21" s="24"/>
-      <c r="C21" s="42"/>
+      <c r="C21" s="41"/>
       <c r="D21" s="49" t="s">
         <v>165</v>
       </c>
@@ -2153,7 +2153,7 @@
     <row r="22">
       <c r="A22" s="24"/>
       <c r="B22" s="24"/>
-      <c r="C22" s="42"/>
+      <c r="C22" s="41"/>
       <c r="D22" s="49" t="s">
         <v>168</v>
       </c>
@@ -2191,7 +2191,7 @@
     <row r="23">
       <c r="A23" s="24"/>
       <c r="B23" s="24"/>
-      <c r="C23" s="42"/>
+      <c r="C23" s="41"/>
       <c r="D23" s="49" t="s">
         <v>172</v>
       </c>
@@ -2229,7 +2229,7 @@
     <row r="24">
       <c r="A24" s="24"/>
       <c r="B24" s="24"/>
-      <c r="C24" s="42"/>
+      <c r="C24" s="41"/>
       <c r="D24" s="49" t="s">
         <v>174</v>
       </c>
@@ -2267,7 +2267,7 @@
     <row r="25">
       <c r="A25" s="24"/>
       <c r="B25" s="24"/>
-      <c r="C25" s="42"/>
+      <c r="C25" s="41"/>
       <c r="D25" s="49" t="s">
         <v>176</v>
       </c>
@@ -2355,7 +2355,7 @@
         <v>46252.0</v>
       </c>
       <c r="H27" s="35" t="s">
-        <v>122</v>
+        <v>126</v>
       </c>
       <c r="I27" s="44"/>
       <c r="J27" s="44">
@@ -2378,34 +2378,34 @@
       <c r="A28" s="24"/>
       <c r="B28" s="24"/>
       <c r="C28" s="29" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="D28" s="29" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="E28" s="30" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="F28" s="30" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="G28" s="30"/>
       <c r="H28" s="30" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="I28" s="30"/>
       <c r="J28" s="30"/>
       <c r="K28" s="30" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="L28" s="30" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="M28" s="30" t="s">
-        <v>67</v>
+        <v>73</v>
       </c>
       <c r="N28" s="30" t="s">
-        <v>68</v>
+        <v>74</v>
       </c>
       <c r="O28" s="26"/>
       <c r="P28" s="28"/>
@@ -2474,7 +2474,7 @@
     <row r="30">
       <c r="A30" s="24"/>
       <c r="B30" s="24"/>
-      <c r="C30" s="42"/>
+      <c r="C30" s="41"/>
       <c r="D30" s="56" t="s">
         <v>186</v>
       </c>
@@ -2523,7 +2523,7 @@
     <row r="31" ht="12.75" customHeight="1">
       <c r="A31" s="24"/>
       <c r="B31" s="24"/>
-      <c r="C31" s="42"/>
+      <c r="C31" s="41"/>
       <c r="D31" s="59" t="s">
         <v>189</v>
       </c>
@@ -2572,7 +2572,7 @@
     <row r="32" ht="60.0" customHeight="1">
       <c r="A32" s="24"/>
       <c r="B32" s="24"/>
-      <c r="C32" s="42"/>
+      <c r="C32" s="41"/>
       <c r="D32" s="59" t="s">
         <v>192</v>
       </c>
@@ -2621,7 +2621,7 @@
     <row r="33" ht="12.75" customHeight="1">
       <c r="A33" s="24"/>
       <c r="B33" s="24"/>
-      <c r="C33" s="42"/>
+      <c r="C33" s="41"/>
       <c r="D33" s="59" t="s">
         <v>194</v>
       </c>
@@ -2635,7 +2635,7 @@
         <v>45904.0</v>
       </c>
       <c r="H33" s="35" t="s">
-        <v>69</v>
+        <v>59</v>
       </c>
       <c r="I33" s="64"/>
       <c r="J33" s="64">
@@ -2670,7 +2670,7 @@
     <row r="34" ht="12.75" customHeight="1">
       <c r="A34" s="24"/>
       <c r="B34" s="24"/>
-      <c r="C34" s="42"/>
+      <c r="C34" s="41"/>
       <c r="D34" s="59" t="s">
         <v>196</v>
       </c>
@@ -2684,7 +2684,7 @@
         <v>46008.0</v>
       </c>
       <c r="H34" s="35" t="s">
-        <v>110</v>
+        <v>114</v>
       </c>
       <c r="I34" s="64"/>
       <c r="J34" s="64">
@@ -2719,7 +2719,7 @@
     <row r="35" ht="12.75" customHeight="1">
       <c r="A35" s="24"/>
       <c r="B35" s="24"/>
-      <c r="C35" s="42"/>
+      <c r="C35" s="41"/>
       <c r="D35" s="59" t="s">
         <v>199</v>
       </c>
@@ -2768,7 +2768,7 @@
     <row r="36" ht="12.75" customHeight="1">
       <c r="A36" s="24"/>
       <c r="B36" s="24"/>
-      <c r="C36" s="42"/>
+      <c r="C36" s="41"/>
       <c r="D36" s="59" t="s">
         <v>203</v>
       </c>
@@ -2782,7 +2782,7 @@
         <v>45968.0</v>
       </c>
       <c r="H36" s="35" t="s">
-        <v>102</v>
+        <v>106</v>
       </c>
       <c r="I36" s="64"/>
       <c r="J36" s="64">
@@ -2817,7 +2817,7 @@
     <row r="37" ht="12.75" customHeight="1">
       <c r="A37" s="24"/>
       <c r="B37" s="24"/>
-      <c r="C37" s="42"/>
+      <c r="C37" s="41"/>
       <c r="D37" s="59" t="s">
         <v>206</v>
       </c>
@@ -2831,7 +2831,7 @@
         <v>46043.0</v>
       </c>
       <c r="H37" s="63" t="s">
-        <v>98</v>
+        <v>101</v>
       </c>
       <c r="I37" s="68"/>
       <c r="J37" s="67">
@@ -2866,7 +2866,7 @@
     <row r="38" ht="12.75" customHeight="1">
       <c r="A38" s="24"/>
       <c r="B38" s="24"/>
-      <c r="C38" s="42"/>
+      <c r="C38" s="41"/>
       <c r="D38" s="59" t="s">
         <v>208</v>
       </c>
@@ -3026,7 +3026,7 @@
         <v>46104.0</v>
       </c>
       <c r="H42" s="63" t="s">
-        <v>98</v>
+        <v>101</v>
       </c>
       <c r="I42" s="68"/>
       <c r="J42" s="67">
@@ -3061,7 +3061,7 @@
     <row r="43" ht="12.75" customHeight="1">
       <c r="A43" s="15"/>
       <c r="B43" s="15"/>
-      <c r="C43" s="42"/>
+      <c r="C43" s="41"/>
       <c r="D43" s="59" t="s">
         <v>216</v>
       </c>
@@ -3073,7 +3073,7 @@
         <v>46199.0</v>
       </c>
       <c r="H43" s="63" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="I43" s="68"/>
       <c r="J43" s="67">
@@ -3083,53 +3083,53 @@
         <v>58868.35</v>
       </c>
       <c r="L43" s="35" t="s">
-        <v>67</v>
+        <v>73</v>
       </c>
       <c r="M43" s="72">
         <v>58868.35</v>
       </c>
       <c r="N43" s="51"/>
-      <c r="V43" s="4"/>
+      <c r="V43" s="5"/>
     </row>
     <row r="44" ht="12.75" customHeight="1">
       <c r="A44" s="15"/>
       <c r="B44" s="15"/>
-      <c r="C44" s="42"/>
+      <c r="C44" s="41"/>
       <c r="K44" s="73"/>
       <c r="M44" s="73"/>
-      <c r="V44" s="4"/>
+      <c r="V44" s="5"/>
     </row>
     <row r="45" ht="12.75" customHeight="1">
       <c r="A45" s="15"/>
       <c r="B45" s="15"/>
-      <c r="C45" s="42"/>
+      <c r="C45" s="41"/>
       <c r="K45" s="73"/>
       <c r="M45" s="73"/>
-      <c r="V45" s="4"/>
+      <c r="V45" s="5"/>
     </row>
     <row r="46" ht="12.75" customHeight="1">
       <c r="A46" s="15"/>
       <c r="B46" s="15"/>
-      <c r="C46" s="42"/>
-      <c r="V46" s="4"/>
+      <c r="C46" s="41"/>
+      <c r="V46" s="5"/>
     </row>
     <row r="47" ht="12.75" customHeight="1">
       <c r="A47" s="15"/>
       <c r="B47" s="15"/>
-      <c r="C47" s="42"/>
-      <c r="V47" s="4"/>
+      <c r="C47" s="41"/>
+      <c r="V47" s="5"/>
     </row>
     <row r="48" ht="12.75" customHeight="1">
       <c r="A48" s="15"/>
       <c r="B48" s="15"/>
-      <c r="C48" s="42"/>
-      <c r="V48" s="4"/>
+      <c r="C48" s="41"/>
+      <c r="V48" s="5"/>
     </row>
     <row r="49" ht="12.75" customHeight="1">
       <c r="A49" s="15"/>
       <c r="B49" s="15"/>
-      <c r="C49" s="42"/>
-      <c r="V49" s="4"/>
+      <c r="C49" s="41"/>
+      <c r="V49" s="5"/>
     </row>
     <row r="50" ht="12.75" customHeight="1">
       <c r="A50" s="15"/>
@@ -3137,7 +3137,7 @@
       <c r="C50" s="55"/>
       <c r="K50" s="73"/>
       <c r="M50" s="73"/>
-      <c r="V50" s="4"/>
+      <c r="V50" s="5"/>
     </row>
     <row r="51" ht="12.75" customHeight="1">
       <c r="A51" s="15"/>
@@ -3161,7 +3161,7 @@
       <c r="S51" s="74"/>
       <c r="T51" s="74"/>
       <c r="U51" s="74"/>
-      <c r="V51" s="4"/>
+      <c r="V51" s="5"/>
     </row>
     <row r="52" ht="12.75" customHeight="1">
       <c r="A52" s="15"/>
@@ -8045,7 +8045,7 @@
       <c r="A2" s="3">
         <v>46258.0</v>
       </c>
-      <c r="L2" s="5" t="s">
+      <c r="L2" s="4" t="s">
         <v>0</v>
       </c>
       <c r="AB2" s="2"/>
@@ -8057,40 +8057,40 @@
       <c r="AH2" s="2"/>
     </row>
     <row r="3">
-      <c r="A3" s="7" t="s">
+      <c r="A3" s="6" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="7" t="s">
-        <v>3</v>
-      </c>
-      <c r="C3" s="9">
+      <c r="B3" s="6" t="s">
+        <v>2</v>
+      </c>
+      <c r="C3" s="8">
         <v>2.5E32</v>
       </c>
-      <c r="D3" s="7" t="s">
+      <c r="D3" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="E3" s="11">
+      <c r="E3" s="9">
         <v>45686.0</v>
       </c>
-      <c r="F3" s="7" t="s">
+      <c r="F3" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="G3" s="7">
+      <c r="G3" s="6">
         <v>12.0</v>
       </c>
-      <c r="H3" s="7">
+      <c r="H3" s="6">
         <v>339039.0</v>
       </c>
-      <c r="I3" s="7">
+      <c r="I3" s="6">
         <v>2048.0</v>
       </c>
-      <c r="J3" s="13">
+      <c r="J3" s="11">
         <v>1000.0</v>
       </c>
-      <c r="K3" s="13">
+      <c r="K3" s="11">
         <v>1000.0</v>
       </c>
-      <c r="L3" s="7">
+      <c r="L3" s="6">
         <v>0.0</v>
       </c>
       <c r="AB3" s="2"/>
@@ -8102,40 +8102,40 @@
       <c r="AH3" s="2"/>
     </row>
     <row r="4">
-      <c r="A4" s="7" t="s">
+      <c r="A4" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="B4" s="7" t="s">
+      <c r="B4" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="C4" s="7" t="s">
+      <c r="C4" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="D4" s="7" t="s">
+      <c r="D4" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="E4" s="11">
+      <c r="E4" s="9">
         <v>45762.0</v>
       </c>
-      <c r="F4" s="7" t="s">
+      <c r="F4" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="G4" s="7">
+      <c r="G4" s="6">
         <v>12.0</v>
       </c>
-      <c r="H4" s="7">
+      <c r="H4" s="6">
         <v>339039.0</v>
       </c>
-      <c r="I4" s="7">
+      <c r="I4" s="6">
         <v>2048.0</v>
       </c>
-      <c r="J4" s="13">
+      <c r="J4" s="11">
         <v>52250.04</v>
       </c>
-      <c r="K4" s="13">
+      <c r="K4" s="11">
         <v>52250.04</v>
       </c>
-      <c r="L4" s="7">
+      <c r="L4" s="6">
         <v>0.0</v>
       </c>
       <c r="AB4" s="2"/>
@@ -8147,40 +8147,40 @@
       <c r="AH4" s="2"/>
     </row>
     <row r="5">
-      <c r="A5" s="7" t="s">
+      <c r="A5" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="B5" s="7" t="s">
+      <c r="B5" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="C5" s="7" t="s">
+      <c r="C5" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="D5" s="7" t="s">
+      <c r="D5" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="E5" s="11">
+      <c r="E5" s="9">
         <v>45762.0</v>
       </c>
-      <c r="F5" s="7" t="s">
+      <c r="F5" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="G5" s="7">
+      <c r="G5" s="6">
         <v>12.0</v>
       </c>
-      <c r="H5" s="7">
+      <c r="H5" s="6">
         <v>339039.0</v>
       </c>
-      <c r="I5" s="7">
+      <c r="I5" s="6">
         <v>2048.0</v>
       </c>
-      <c r="J5" s="13">
+      <c r="J5" s="11">
         <v>881914.18</v>
       </c>
-      <c r="K5" s="13">
+      <c r="K5" s="11">
         <v>881914.18</v>
       </c>
-      <c r="L5" s="7">
+      <c r="L5" s="6">
         <v>0.0</v>
       </c>
       <c r="AB5" s="2"/>
@@ -8192,40 +8192,40 @@
       <c r="AH5" s="2"/>
     </row>
     <row r="6">
-      <c r="A6" s="7" t="s">
-        <v>25</v>
-      </c>
-      <c r="B6" s="7" t="s">
+      <c r="A6" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="B6" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="C6" s="7" t="s">
-        <v>27</v>
-      </c>
-      <c r="D6" s="7" t="s">
+      <c r="C6" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="D6" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="E6" s="11">
+      <c r="E6" s="9">
         <v>45762.0</v>
       </c>
-      <c r="F6" s="7" t="s">
+      <c r="F6" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="G6" s="7">
+      <c r="G6" s="6">
         <v>12.0</v>
       </c>
-      <c r="H6" s="7">
+      <c r="H6" s="6">
         <v>339039.0</v>
       </c>
-      <c r="I6" s="7">
+      <c r="I6" s="6">
         <v>2048.0</v>
       </c>
-      <c r="J6" s="13">
+      <c r="J6" s="11">
         <v>750000.0</v>
       </c>
-      <c r="K6" s="13">
+      <c r="K6" s="11">
         <v>750000.0</v>
       </c>
-      <c r="L6" s="7">
+      <c r="L6" s="6">
         <v>0.0</v>
       </c>
       <c r="AB6" s="2"/>
@@ -8237,40 +8237,40 @@
       <c r="AH6" s="2"/>
     </row>
     <row r="7">
-      <c r="A7" s="7" t="s">
-        <v>33</v>
-      </c>
-      <c r="B7" s="7" t="s">
-        <v>34</v>
-      </c>
-      <c r="C7" s="7" t="s">
-        <v>35</v>
-      </c>
-      <c r="D7" s="7" t="s">
+      <c r="A7" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="B7" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="C7" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="D7" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="E7" s="11">
+      <c r="E7" s="9">
         <v>45763.0</v>
       </c>
-      <c r="F7" s="7" t="s">
+      <c r="F7" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="G7" s="7">
+      <c r="G7" s="6">
         <v>12.0</v>
       </c>
-      <c r="H7" s="7">
+      <c r="H7" s="6">
         <v>339039.0</v>
       </c>
-      <c r="I7" s="7" t="s">
-        <v>39</v>
-      </c>
-      <c r="J7" s="13">
+      <c r="I7" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="J7" s="11">
         <v>949835.78</v>
       </c>
-      <c r="K7" s="13">
+      <c r="K7" s="11">
         <v>949835.78</v>
       </c>
-      <c r="L7" s="7">
+      <c r="L7" s="6">
         <v>0.0</v>
       </c>
       <c r="AB7" s="2"/>
@@ -8282,43 +8282,43 @@
       <c r="AH7" s="2"/>
     </row>
     <row r="8">
-      <c r="A8" s="7" t="s">
-        <v>40</v>
-      </c>
-      <c r="B8" s="7" t="s">
+      <c r="A8" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="B8" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="C8" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="D8" s="6" t="s">
+        <v>4</v>
+      </c>
+      <c r="E8" s="9">
+        <v>45763.0</v>
+      </c>
+      <c r="F8" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="G8" s="6">
+        <v>12.0</v>
+      </c>
+      <c r="H8" s="6">
+        <v>339039.0</v>
+      </c>
+      <c r="I8" s="6" t="s">
         <v>41</v>
       </c>
-      <c r="C8" s="7" t="s">
-        <v>43</v>
-      </c>
-      <c r="D8" s="7" t="s">
-        <v>4</v>
-      </c>
-      <c r="E8" s="11">
-        <v>45763.0</v>
-      </c>
-      <c r="F8" s="7" t="s">
-        <v>5</v>
-      </c>
-      <c r="G8" s="7">
-        <v>12.0</v>
-      </c>
-      <c r="H8" s="7">
-        <v>339039.0</v>
-      </c>
-      <c r="I8" s="7" t="s">
-        <v>47</v>
-      </c>
-      <c r="J8" s="13">
+      <c r="J8" s="11">
         <v>524584.95</v>
       </c>
-      <c r="K8" s="13">
+      <c r="K8" s="11">
         <v>524584.95</v>
       </c>
-      <c r="L8" s="7">
+      <c r="L8" s="6">
         <v>0.0</v>
       </c>
-      <c r="O8" s="22"/>
+      <c r="O8" s="21"/>
       <c r="AB8" s="2"/>
       <c r="AC8" s="2"/>
       <c r="AD8" s="2"/>
@@ -8328,40 +8328,40 @@
       <c r="AH8" s="2"/>
     </row>
     <row r="9">
-      <c r="A9" s="7" t="s">
+      <c r="A9" s="6" t="s">
         <v>49</v>
       </c>
-      <c r="B9" s="7" t="s">
+      <c r="B9" s="6" t="s">
         <v>50</v>
       </c>
-      <c r="C9" s="7" t="s">
+      <c r="C9" s="6" t="s">
         <v>51</v>
       </c>
-      <c r="D9" s="7" t="s">
+      <c r="D9" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="E9" s="11">
+      <c r="E9" s="9">
         <v>45792.0</v>
       </c>
-      <c r="F9" s="7" t="s">
+      <c r="F9" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="G9" s="7">
+      <c r="G9" s="6">
         <v>12.0</v>
       </c>
-      <c r="H9" s="7">
+      <c r="H9" s="6">
         <v>339039.0</v>
       </c>
-      <c r="I9" s="7" t="s">
+      <c r="I9" s="6" t="s">
         <v>52</v>
       </c>
-      <c r="J9" s="13">
+      <c r="J9" s="11">
         <v>211614.23</v>
       </c>
-      <c r="K9" s="13">
+      <c r="K9" s="11">
         <v>211614.23</v>
       </c>
-      <c r="L9" s="7">
+      <c r="L9" s="6">
         <v>0.0</v>
       </c>
       <c r="AB9" s="2"/>
@@ -8373,40 +8373,40 @@
       <c r="AH9" s="2"/>
     </row>
     <row r="10">
-      <c r="A10" s="7" t="s">
+      <c r="A10" s="6" t="s">
         <v>53</v>
       </c>
-      <c r="B10" s="7" t="s">
+      <c r="B10" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="C10" s="7" t="s">
+      <c r="C10" s="6" t="s">
         <v>54</v>
       </c>
-      <c r="D10" s="7" t="s">
+      <c r="D10" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="E10" s="11">
+      <c r="E10" s="9">
         <v>45825.0</v>
       </c>
-      <c r="F10" s="7" t="s">
+      <c r="F10" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="G10" s="7">
+      <c r="G10" s="6">
         <v>12.0</v>
       </c>
-      <c r="H10" s="7">
+      <c r="H10" s="6">
         <v>339039.0</v>
       </c>
-      <c r="I10" s="7">
+      <c r="I10" s="6">
         <v>2048.0</v>
       </c>
-      <c r="J10" s="13">
+      <c r="J10" s="11">
         <v>2391157.42</v>
       </c>
-      <c r="K10" s="13">
+      <c r="K10" s="11">
         <v>2391157.41</v>
       </c>
-      <c r="L10" s="13">
+      <c r="L10" s="11">
         <v>0.01</v>
       </c>
       <c r="AB10" s="2"/>
@@ -8418,40 +8418,40 @@
       <c r="AH10" s="2"/>
     </row>
     <row r="11">
-      <c r="A11" s="7" t="s">
-        <v>57</v>
-      </c>
-      <c r="B11" s="7" t="s">
+      <c r="A11" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="B11" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="C11" s="7" t="s">
-        <v>58</v>
-      </c>
-      <c r="D11" s="7" t="s">
+      <c r="C11" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="D11" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="E11" s="11">
+      <c r="E11" s="9">
         <v>45825.0</v>
       </c>
-      <c r="F11" s="7" t="s">
+      <c r="F11" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="G11" s="7">
+      <c r="G11" s="6">
         <v>12.0</v>
       </c>
-      <c r="H11" s="7">
+      <c r="H11" s="6">
         <v>339039.0</v>
       </c>
-      <c r="I11" s="7">
+      <c r="I11" s="6">
         <v>2048.0</v>
       </c>
-      <c r="J11" s="13">
+      <c r="J11" s="11">
         <v>618154.39</v>
       </c>
-      <c r="K11" s="13">
+      <c r="K11" s="11">
         <v>618154.38</v>
       </c>
-      <c r="L11" s="7">
+      <c r="L11" s="6">
         <v>0.01</v>
       </c>
       <c r="AB11" s="2"/>
@@ -8463,40 +8463,40 @@
       <c r="AH11" s="2"/>
     </row>
     <row r="12">
-      <c r="A12" s="7" t="s">
-        <v>69</v>
-      </c>
-      <c r="B12" s="7" t="s">
-        <v>70</v>
-      </c>
-      <c r="C12" s="7" t="s">
-        <v>71</v>
-      </c>
-      <c r="D12" s="7" t="s">
+      <c r="A12" s="6" t="s">
+        <v>59</v>
+      </c>
+      <c r="B12" s="6" t="s">
+        <v>60</v>
+      </c>
+      <c r="C12" s="6" t="s">
+        <v>62</v>
+      </c>
+      <c r="D12" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="E12" s="11">
+      <c r="E12" s="9">
         <v>45832.0</v>
       </c>
-      <c r="F12" s="7" t="s">
+      <c r="F12" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="G12" s="7">
+      <c r="G12" s="6">
         <v>12.0</v>
       </c>
-      <c r="H12" s="7">
+      <c r="H12" s="6">
         <v>339039.0</v>
       </c>
-      <c r="I12" s="7" t="s">
-        <v>72</v>
-      </c>
-      <c r="J12" s="13">
+      <c r="I12" s="6" t="s">
+        <v>65</v>
+      </c>
+      <c r="J12" s="11">
         <v>1600334.09</v>
       </c>
-      <c r="K12" s="13">
+      <c r="K12" s="11">
         <v>1600334.09</v>
       </c>
-      <c r="L12" s="7">
+      <c r="L12" s="6">
         <v>0.0</v>
       </c>
       <c r="AB12" s="2"/>
@@ -8508,40 +8508,40 @@
       <c r="AH12" s="2"/>
     </row>
     <row r="13">
-      <c r="A13" s="7" t="s">
-        <v>73</v>
-      </c>
-      <c r="B13" s="7" t="s">
+      <c r="A13" s="6" t="s">
+        <v>71</v>
+      </c>
+      <c r="B13" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="C13" s="7" t="s">
-        <v>74</v>
-      </c>
-      <c r="D13" s="7" t="s">
+      <c r="C13" s="6" t="s">
+        <v>72</v>
+      </c>
+      <c r="D13" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="E13" s="11">
+      <c r="E13" s="9">
         <v>45863.0</v>
       </c>
-      <c r="F13" s="7" t="s">
+      <c r="F13" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="G13" s="7">
+      <c r="G13" s="6">
         <v>12.0</v>
       </c>
-      <c r="H13" s="7">
+      <c r="H13" s="6">
         <v>339039.0</v>
       </c>
-      <c r="I13" s="7">
+      <c r="I13" s="6">
         <v>2048.0</v>
       </c>
-      <c r="J13" s="13">
+      <c r="J13" s="11">
         <v>2364771.07</v>
       </c>
-      <c r="K13" s="13">
+      <c r="K13" s="11">
         <v>2364771.07</v>
       </c>
-      <c r="L13" s="13">
+      <c r="L13" s="11">
         <v>0.0</v>
       </c>
       <c r="M13" s="32"/>
@@ -8554,40 +8554,40 @@
       <c r="AH13" s="2"/>
     </row>
     <row r="14">
-      <c r="A14" s="7" t="s">
+      <c r="A14" s="6" t="s">
         <v>75</v>
       </c>
-      <c r="B14" s="7" t="s">
+      <c r="B14" s="6" t="s">
         <v>76</v>
       </c>
-      <c r="C14" s="7" t="s">
+      <c r="C14" s="6" t="s">
         <v>77</v>
       </c>
-      <c r="D14" s="7" t="s">
+      <c r="D14" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="E14" s="11">
+      <c r="E14" s="9">
         <v>45887.0</v>
       </c>
-      <c r="F14" s="7" t="s">
+      <c r="F14" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="G14" s="7">
+      <c r="G14" s="6">
         <v>12.0</v>
       </c>
-      <c r="H14" s="7">
+      <c r="H14" s="6">
         <v>339039.0</v>
       </c>
-      <c r="I14" s="7" t="s">
+      <c r="I14" s="6" t="s">
         <v>52</v>
       </c>
-      <c r="J14" s="13">
+      <c r="J14" s="11">
         <v>968237.39</v>
       </c>
-      <c r="K14" s="13">
+      <c r="K14" s="11">
         <v>968237.39</v>
       </c>
-      <c r="L14" s="7">
+      <c r="L14" s="6">
         <v>0.0</v>
       </c>
       <c r="AB14" s="2"/>
@@ -8599,40 +8599,40 @@
       <c r="AH14" s="2"/>
     </row>
     <row r="15">
-      <c r="A15" s="7" t="s">
+      <c r="A15" s="6" t="s">
         <v>79</v>
       </c>
-      <c r="B15" s="7" t="s">
+      <c r="B15" s="6" t="s">
         <v>80</v>
       </c>
-      <c r="C15" s="7" t="s">
+      <c r="C15" s="6" t="s">
         <v>82</v>
       </c>
-      <c r="D15" s="7" t="s">
+      <c r="D15" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="E15" s="11">
+      <c r="E15" s="9">
         <v>45924.0</v>
       </c>
-      <c r="F15" s="7" t="s">
+      <c r="F15" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="G15" s="7">
+      <c r="G15" s="6">
         <v>12.0</v>
       </c>
-      <c r="H15" s="7">
+      <c r="H15" s="6">
         <v>339039.0</v>
       </c>
-      <c r="I15" s="7" t="s">
-        <v>39</v>
-      </c>
-      <c r="J15" s="13">
+      <c r="I15" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="J15" s="11">
         <v>1011677.95</v>
       </c>
-      <c r="K15" s="13">
+      <c r="K15" s="11">
         <v>1011677.95</v>
       </c>
-      <c r="L15" s="7">
+      <c r="L15" s="6">
         <v>0.0</v>
       </c>
       <c r="AB15" s="2"/>
@@ -8644,40 +8644,40 @@
       <c r="AH15" s="2"/>
     </row>
     <row r="16">
-      <c r="A16" s="7" t="s">
+      <c r="A16" s="6" t="s">
+        <v>84</v>
+      </c>
+      <c r="B16" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="C16" s="6" t="s">
         <v>85</v>
       </c>
-      <c r="B16" s="7" t="s">
-        <v>7</v>
-      </c>
-      <c r="C16" s="7" t="s">
-        <v>86</v>
-      </c>
-      <c r="D16" s="7" t="s">
+      <c r="D16" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="E16" s="11">
+      <c r="E16" s="9">
         <v>45929.0</v>
       </c>
-      <c r="F16" s="7" t="s">
+      <c r="F16" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="G16" s="7">
+      <c r="G16" s="6">
         <v>12.0</v>
       </c>
-      <c r="H16" s="7">
+      <c r="H16" s="6">
         <v>339039.0</v>
       </c>
-      <c r="I16" s="7">
+      <c r="I16" s="6">
         <v>2048.0</v>
       </c>
-      <c r="J16" s="13">
+      <c r="J16" s="11">
         <v>1580293.02</v>
       </c>
-      <c r="K16" s="13">
+      <c r="K16" s="11">
         <v>1580293.02</v>
       </c>
-      <c r="L16" s="13">
+      <c r="L16" s="11">
         <v>0.0</v>
       </c>
       <c r="AB16" s="2"/>
@@ -8689,40 +8689,40 @@
       <c r="AH16" s="2"/>
     </row>
     <row r="17">
-      <c r="A17" s="7" t="s">
+      <c r="A17" s="6" t="s">
         <v>87</v>
       </c>
-      <c r="B17" s="7" t="s">
+      <c r="B17" s="6" t="s">
         <v>88</v>
       </c>
-      <c r="C17" s="7" t="s">
+      <c r="C17" s="6" t="s">
         <v>89</v>
       </c>
-      <c r="D17" s="7" t="s">
+      <c r="D17" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="E17" s="11">
+      <c r="E17" s="9">
         <v>45930.0</v>
       </c>
-      <c r="F17" s="7" t="s">
+      <c r="F17" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="G17" s="7">
+      <c r="G17" s="6">
         <v>12.0</v>
       </c>
-      <c r="H17" s="7">
+      <c r="H17" s="6">
         <v>339039.0</v>
       </c>
-      <c r="I17" s="7">
+      <c r="I17" s="6">
         <v>2048.0</v>
       </c>
-      <c r="J17" s="13">
+      <c r="J17" s="11">
         <v>34065.36</v>
       </c>
-      <c r="K17" s="7">
+      <c r="K17" s="6">
         <v>0.0</v>
       </c>
-      <c r="L17" s="13">
+      <c r="L17" s="11">
         <v>34065.36</v>
       </c>
       <c r="AB17" s="2"/>
@@ -8734,40 +8734,40 @@
       <c r="AH17" s="2"/>
     </row>
     <row r="18">
-      <c r="A18" s="7" t="s">
+      <c r="A18" s="6" t="s">
         <v>90</v>
       </c>
-      <c r="B18" s="7" t="s">
+      <c r="B18" s="6" t="s">
         <v>76</v>
       </c>
-      <c r="C18" s="7" t="s">
+      <c r="C18" s="6" t="s">
         <v>91</v>
       </c>
-      <c r="D18" s="7" t="s">
+      <c r="D18" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="E18" s="11">
+      <c r="E18" s="9">
         <v>45938.0</v>
       </c>
-      <c r="F18" s="7" t="s">
+      <c r="F18" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="G18" s="7">
+      <c r="G18" s="6">
         <v>12.0</v>
       </c>
-      <c r="H18" s="7">
+      <c r="H18" s="6">
         <v>339039.0</v>
       </c>
-      <c r="I18" s="7" t="s">
+      <c r="I18" s="6" t="s">
         <v>52</v>
       </c>
-      <c r="J18" s="13">
+      <c r="J18" s="11">
         <v>63746.85</v>
       </c>
-      <c r="K18" s="13">
+      <c r="K18" s="11">
         <v>63746.85</v>
       </c>
-      <c r="L18" s="7">
+      <c r="L18" s="6">
         <v>0.0</v>
       </c>
       <c r="AB18" s="2"/>
@@ -8779,40 +8779,40 @@
       <c r="AH18" s="2"/>
     </row>
     <row r="19">
-      <c r="A19" s="7" t="s">
+      <c r="A19" s="6" t="s">
         <v>92</v>
       </c>
-      <c r="B19" s="7" t="s">
-        <v>70</v>
-      </c>
-      <c r="C19" s="7" t="s">
+      <c r="B19" s="6" t="s">
+        <v>60</v>
+      </c>
+      <c r="C19" s="6" t="s">
         <v>93</v>
       </c>
-      <c r="D19" s="7" t="s">
+      <c r="D19" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="E19" s="11">
+      <c r="E19" s="9">
         <v>45938.0</v>
       </c>
-      <c r="F19" s="7" t="s">
+      <c r="F19" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="G19" s="7">
+      <c r="G19" s="6">
         <v>12.0</v>
       </c>
-      <c r="H19" s="7">
+      <c r="H19" s="6">
         <v>339039.0</v>
       </c>
-      <c r="I19" s="7" t="s">
-        <v>72</v>
-      </c>
-      <c r="J19" s="13">
+      <c r="I19" s="6" t="s">
+        <v>65</v>
+      </c>
+      <c r="J19" s="11">
         <v>947931.1</v>
       </c>
-      <c r="K19" s="13">
+      <c r="K19" s="11">
         <v>947931.1</v>
       </c>
-      <c r="L19" s="7">
+      <c r="L19" s="6">
         <v>0.0</v>
       </c>
       <c r="AB19" s="2"/>
@@ -8824,40 +8824,40 @@
       <c r="AH19" s="2"/>
     </row>
     <row r="20">
-      <c r="A20" s="7" t="s">
+      <c r="A20" s="6" t="s">
         <v>94</v>
       </c>
-      <c r="B20" s="7" t="s">
+      <c r="B20" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="C20" s="7" t="s">
+      <c r="C20" s="6" t="s">
         <v>95</v>
       </c>
-      <c r="D20" s="7" t="s">
+      <c r="D20" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="E20" s="11">
+      <c r="E20" s="9">
         <v>45938.0</v>
       </c>
-      <c r="F20" s="7" t="s">
+      <c r="F20" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="G20" s="7">
+      <c r="G20" s="6">
         <v>12.0</v>
       </c>
-      <c r="H20" s="7">
+      <c r="H20" s="6">
         <v>339039.0</v>
       </c>
-      <c r="I20" s="7">
+      <c r="I20" s="6">
         <v>2048.0</v>
       </c>
-      <c r="J20" s="13">
+      <c r="J20" s="11">
         <v>259790.57</v>
       </c>
-      <c r="K20" s="13">
+      <c r="K20" s="11">
         <v>259790.57</v>
       </c>
-      <c r="L20" s="7">
+      <c r="L20" s="6">
         <v>0.0</v>
       </c>
       <c r="AB20" s="2"/>
@@ -8869,40 +8869,40 @@
       <c r="AH20" s="2"/>
     </row>
     <row r="21">
-      <c r="A21" s="7" t="s">
-        <v>96</v>
-      </c>
-      <c r="B21" s="7" t="s">
+      <c r="A21" s="6" t="s">
+        <v>97</v>
+      </c>
+      <c r="B21" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="C21" s="7" t="s">
-        <v>97</v>
-      </c>
-      <c r="D21" s="7" t="s">
+      <c r="C21" s="6" t="s">
+        <v>98</v>
+      </c>
+      <c r="D21" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="E21" s="11">
+      <c r="E21" s="9">
         <v>45938.0</v>
       </c>
-      <c r="F21" s="7" t="s">
+      <c r="F21" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="G21" s="7">
+      <c r="G21" s="6">
         <v>12.0</v>
       </c>
-      <c r="H21" s="7">
+      <c r="H21" s="6">
         <v>339039.0</v>
       </c>
-      <c r="I21" s="7">
+      <c r="I21" s="6">
         <v>2048.0</v>
       </c>
-      <c r="J21" s="13">
+      <c r="J21" s="11">
         <v>170479.3</v>
       </c>
-      <c r="K21" s="13">
+      <c r="K21" s="11">
         <v>170479.3</v>
       </c>
-      <c r="L21" s="7">
+      <c r="L21" s="6">
         <v>0.0</v>
       </c>
       <c r="AB21" s="2"/>
@@ -8914,40 +8914,40 @@
       <c r="AH21" s="2"/>
     </row>
     <row r="22">
-      <c r="A22" s="7" t="s">
-        <v>98</v>
-      </c>
-      <c r="B22" s="7" t="s">
-        <v>99</v>
-      </c>
-      <c r="C22" s="7" t="s">
-        <v>100</v>
-      </c>
-      <c r="D22" s="7" t="s">
+      <c r="A22" s="6" t="s">
+        <v>101</v>
+      </c>
+      <c r="B22" s="6" t="s">
+        <v>102</v>
+      </c>
+      <c r="C22" s="6" t="s">
+        <v>103</v>
+      </c>
+      <c r="D22" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="E22" s="41">
+      <c r="E22" s="43">
         <v>45953.0</v>
       </c>
-      <c r="F22" s="7" t="s">
+      <c r="F22" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="G22" s="7">
+      <c r="G22" s="6">
         <v>12.0</v>
       </c>
-      <c r="H22" s="7">
+      <c r="H22" s="6">
         <v>339039.0</v>
       </c>
-      <c r="I22" s="7">
+      <c r="I22" s="6">
         <v>2000.0</v>
       </c>
-      <c r="J22" s="13">
+      <c r="J22" s="11">
         <v>1500000.0</v>
       </c>
-      <c r="K22" s="13">
+      <c r="K22" s="11">
         <v>1500000.0</v>
       </c>
-      <c r="L22" s="13">
+      <c r="L22" s="11">
         <v>0.0</v>
       </c>
       <c r="AB22" s="2"/>
@@ -8959,40 +8959,40 @@
       <c r="AH22" s="2"/>
     </row>
     <row r="23">
-      <c r="A23" s="7" t="s">
-        <v>102</v>
-      </c>
-      <c r="B23" s="7" t="s">
-        <v>103</v>
-      </c>
-      <c r="C23" s="7" t="s">
-        <v>104</v>
-      </c>
-      <c r="D23" s="7" t="s">
+      <c r="A23" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="B23" s="6" t="s">
+        <v>108</v>
+      </c>
+      <c r="C23" s="6" t="s">
+        <v>109</v>
+      </c>
+      <c r="D23" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="E23" s="41">
+      <c r="E23" s="43">
         <v>45953.0</v>
       </c>
-      <c r="F23" s="7" t="s">
+      <c r="F23" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="G23" s="7">
+      <c r="G23" s="6">
         <v>12.0</v>
       </c>
-      <c r="H23" s="7">
+      <c r="H23" s="6">
         <v>339039.0</v>
       </c>
-      <c r="I23" s="7" t="s">
-        <v>106</v>
-      </c>
-      <c r="J23" s="13">
+      <c r="I23" s="6" t="s">
+        <v>110</v>
+      </c>
+      <c r="J23" s="11">
         <v>1000001.64</v>
       </c>
-      <c r="K23" s="13">
+      <c r="K23" s="11">
         <v>1000001.64</v>
       </c>
-      <c r="L23" s="7">
+      <c r="L23" s="6">
         <v>0.0</v>
       </c>
       <c r="AB23" s="2"/>
@@ -9004,40 +9004,40 @@
       <c r="AH23" s="2"/>
     </row>
     <row r="24">
-      <c r="A24" s="7" t="s">
-        <v>108</v>
-      </c>
-      <c r="B24" s="7" t="s">
+      <c r="A24" s="6" t="s">
+        <v>112</v>
+      </c>
+      <c r="B24" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="C24" s="7" t="s">
-        <v>109</v>
-      </c>
-      <c r="D24" s="7" t="s">
+      <c r="C24" s="6" t="s">
+        <v>113</v>
+      </c>
+      <c r="D24" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="E24" s="41">
+      <c r="E24" s="43">
         <v>45953.0</v>
       </c>
-      <c r="F24" s="7" t="s">
+      <c r="F24" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="G24" s="7">
+      <c r="G24" s="6">
         <v>12.0</v>
       </c>
-      <c r="H24" s="7">
+      <c r="H24" s="6">
         <v>339039.0</v>
       </c>
-      <c r="I24" s="7">
+      <c r="I24" s="6">
         <v>2048.0</v>
       </c>
-      <c r="J24" s="13">
+      <c r="J24" s="11">
         <v>68405.66</v>
       </c>
-      <c r="K24" s="13">
+      <c r="K24" s="11">
         <v>68405.66</v>
       </c>
-      <c r="L24" s="7">
+      <c r="L24" s="6">
         <v>0.0</v>
       </c>
       <c r="AB24" s="2"/>
@@ -9049,40 +9049,40 @@
       <c r="AH24" s="2"/>
     </row>
     <row r="25">
-      <c r="A25" s="7" t="s">
+      <c r="A25" s="6" t="s">
+        <v>114</v>
+      </c>
+      <c r="B25" s="6" t="s">
+        <v>115</v>
+      </c>
+      <c r="C25" s="6" t="s">
+        <v>116</v>
+      </c>
+      <c r="D25" s="6" t="s">
+        <v>4</v>
+      </c>
+      <c r="E25" s="43">
+        <v>45975.0</v>
+      </c>
+      <c r="F25" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="G25" s="6">
+        <v>12.0</v>
+      </c>
+      <c r="H25" s="6">
+        <v>339039.0</v>
+      </c>
+      <c r="I25" s="6" t="s">
         <v>110</v>
       </c>
-      <c r="B25" s="7" t="s">
-        <v>111</v>
-      </c>
-      <c r="C25" s="7" t="s">
-        <v>112</v>
-      </c>
-      <c r="D25" s="7" t="s">
-        <v>4</v>
-      </c>
-      <c r="E25" s="41">
-        <v>45975.0</v>
-      </c>
-      <c r="F25" s="7" t="s">
-        <v>5</v>
-      </c>
-      <c r="G25" s="7">
-        <v>12.0</v>
-      </c>
-      <c r="H25" s="7">
-        <v>339039.0</v>
-      </c>
-      <c r="I25" s="7" t="s">
-        <v>106</v>
-      </c>
-      <c r="J25" s="13">
+      <c r="J25" s="11">
         <v>1157673.06</v>
       </c>
-      <c r="K25" s="13">
+      <c r="K25" s="11">
         <v>1157673.06</v>
       </c>
-      <c r="L25" s="7">
+      <c r="L25" s="6">
         <v>0.0</v>
       </c>
       <c r="AB25" s="2"/>
@@ -9094,40 +9094,40 @@
       <c r="AH25" s="2"/>
     </row>
     <row r="26">
-      <c r="A26" s="7" t="s">
-        <v>114</v>
-      </c>
-      <c r="B26" s="7" t="s">
+      <c r="A26" s="6" t="s">
+        <v>118</v>
+      </c>
+      <c r="B26" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="C26" s="7" t="s">
-        <v>116</v>
-      </c>
-      <c r="D26" s="7" t="s">
+      <c r="C26" s="6" t="s">
+        <v>119</v>
+      </c>
+      <c r="D26" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="E26" s="41">
+      <c r="E26" s="43">
         <v>45989.0</v>
       </c>
-      <c r="F26" s="7" t="s">
+      <c r="F26" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="G26" s="7">
+      <c r="G26" s="6">
         <v>12.0</v>
       </c>
-      <c r="H26" s="7">
+      <c r="H26" s="6">
         <v>339039.0</v>
       </c>
-      <c r="I26" s="7">
+      <c r="I26" s="6">
         <v>2048.0</v>
       </c>
-      <c r="J26" s="13">
+      <c r="J26" s="11">
         <v>34065.36</v>
       </c>
-      <c r="K26" s="13">
+      <c r="K26" s="11">
         <v>34065.36</v>
       </c>
-      <c r="L26" s="7">
+      <c r="L26" s="6">
         <v>0.0</v>
       </c>
       <c r="AB26" s="2"/>
@@ -9139,40 +9139,40 @@
       <c r="AH26" s="2"/>
     </row>
     <row r="27">
-      <c r="A27" s="7" t="s">
-        <v>118</v>
-      </c>
-      <c r="B27" s="7" t="s">
-        <v>119</v>
-      </c>
-      <c r="C27" s="7" t="s">
-        <v>120</v>
-      </c>
-      <c r="D27" s="7" t="s">
+      <c r="A27" s="6" t="s">
+        <v>121</v>
+      </c>
+      <c r="B27" s="6" t="s">
+        <v>122</v>
+      </c>
+      <c r="C27" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="D27" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="E27" s="11">
+      <c r="E27" s="9">
         <v>46104.0</v>
       </c>
-      <c r="F27" s="7" t="s">
+      <c r="F27" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="G27" s="7">
+      <c r="G27" s="6">
         <v>12.0</v>
       </c>
-      <c r="H27" s="7">
+      <c r="H27" s="6">
         <v>339039.0</v>
       </c>
-      <c r="I27" s="7">
+      <c r="I27" s="6">
         <v>2048.0</v>
       </c>
-      <c r="J27" s="13">
+      <c r="J27" s="11">
         <v>1770880.5</v>
       </c>
-      <c r="K27" s="13">
+      <c r="K27" s="11">
         <v>843261.89</v>
       </c>
-      <c r="L27" s="13">
+      <c r="L27" s="11">
         <v>927618.61</v>
       </c>
       <c r="AB27" s="2"/>
@@ -9184,40 +9184,40 @@
       <c r="AH27" s="2"/>
     </row>
     <row r="28">
-      <c r="A28" s="7" t="s">
-        <v>122</v>
-      </c>
-      <c r="B28" s="7" t="s">
-        <v>123</v>
-      </c>
-      <c r="C28" s="7" t="s">
-        <v>124</v>
-      </c>
-      <c r="D28" s="7" t="s">
+      <c r="A28" s="6" t="s">
+        <v>126</v>
+      </c>
+      <c r="B28" s="6" t="s">
+        <v>128</v>
+      </c>
+      <c r="C28" s="6" t="s">
+        <v>129</v>
+      </c>
+      <c r="D28" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="E28" s="11">
+      <c r="E28" s="9">
         <v>46120.0</v>
       </c>
-      <c r="F28" s="7" t="s">
+      <c r="F28" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="G28" s="7">
+      <c r="G28" s="6">
         <v>12.0</v>
       </c>
-      <c r="H28" s="7">
+      <c r="H28" s="6">
         <v>339039.0</v>
       </c>
-      <c r="I28" s="7" t="s">
-        <v>47</v>
-      </c>
-      <c r="J28" s="13">
+      <c r="I28" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="J28" s="11">
         <v>1912292.52</v>
       </c>
-      <c r="K28" s="13">
+      <c r="K28" s="11">
         <v>1629834.48</v>
       </c>
-      <c r="L28" s="13">
+      <c r="L28" s="11">
         <v>282458.04</v>
       </c>
       <c r="AB28" s="2"/>
@@ -9229,40 +9229,40 @@
       <c r="AH28" s="2"/>
     </row>
     <row r="29">
-      <c r="A29" s="7" t="s">
-        <v>126</v>
-      </c>
-      <c r="B29" s="7" t="s">
-        <v>127</v>
-      </c>
-      <c r="C29" s="7" t="s">
-        <v>128</v>
-      </c>
-      <c r="D29" s="7" t="s">
+      <c r="A29" s="6" t="s">
+        <v>133</v>
+      </c>
+      <c r="B29" s="6" t="s">
+        <v>134</v>
+      </c>
+      <c r="C29" s="6" t="s">
+        <v>135</v>
+      </c>
+      <c r="D29" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="E29" s="11">
+      <c r="E29" s="9">
         <v>46196.0</v>
       </c>
-      <c r="F29" s="7" t="s">
+      <c r="F29" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="G29" s="7">
+      <c r="G29" s="6">
         <v>12.0</v>
       </c>
-      <c r="H29" s="7">
+      <c r="H29" s="6">
         <v>339039.0</v>
       </c>
-      <c r="I29" s="7">
+      <c r="I29" s="6">
         <v>2048.0</v>
       </c>
-      <c r="J29" s="13">
+      <c r="J29" s="11">
         <v>1496713.48</v>
       </c>
-      <c r="K29" s="7">
+      <c r="K29" s="6">
         <v>0.0</v>
       </c>
-      <c r="L29" s="13">
+      <c r="L29" s="11">
         <v>1496713.48</v>
       </c>
       <c r="AB29" s="2"/>
@@ -9274,40 +9274,40 @@
       <c r="AH29" s="2"/>
     </row>
     <row r="30">
-      <c r="A30" s="7" t="s">
-        <v>129</v>
-      </c>
-      <c r="B30" s="7" t="s">
-        <v>130</v>
-      </c>
-      <c r="C30" s="7" t="s">
-        <v>131</v>
-      </c>
-      <c r="D30" s="7" t="s">
+      <c r="A30" s="6" t="s">
+        <v>138</v>
+      </c>
+      <c r="B30" s="6" t="s">
+        <v>140</v>
+      </c>
+      <c r="C30" s="6" t="s">
+        <v>141</v>
+      </c>
+      <c r="D30" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="E30" s="11">
+      <c r="E30" s="9">
         <v>46205.0</v>
       </c>
-      <c r="F30" s="7" t="s">
+      <c r="F30" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="G30" s="7">
+      <c r="G30" s="6">
         <v>12.0</v>
       </c>
-      <c r="H30" s="7">
+      <c r="H30" s="6">
         <v>339039.0</v>
       </c>
-      <c r="I30" s="7" t="s">
-        <v>39</v>
-      </c>
-      <c r="J30" s="13">
+      <c r="I30" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="J30" s="11">
         <v>624166.14</v>
       </c>
-      <c r="K30" s="7">
+      <c r="K30" s="6">
         <v>0.0</v>
       </c>
-      <c r="L30" s="13">
+      <c r="L30" s="11">
         <v>624166.14</v>
       </c>
       <c r="AB30" s="2"/>
@@ -9319,40 +9319,40 @@
       <c r="AH30" s="2"/>
     </row>
     <row r="31">
-      <c r="A31" s="7" t="s">
-        <v>133</v>
-      </c>
-      <c r="B31" s="7" t="s">
-        <v>134</v>
-      </c>
-      <c r="C31" s="7" t="s">
-        <v>135</v>
-      </c>
-      <c r="D31" s="7" t="s">
+      <c r="A31" s="6" t="s">
+        <v>146</v>
+      </c>
+      <c r="B31" s="6" t="s">
+        <v>147</v>
+      </c>
+      <c r="C31" s="6" t="s">
+        <v>148</v>
+      </c>
+      <c r="D31" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="E31" s="11">
+      <c r="E31" s="9">
         <v>46205.0</v>
       </c>
-      <c r="F31" s="7" t="s">
+      <c r="F31" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="G31" s="7">
+      <c r="G31" s="6">
         <v>12.0</v>
       </c>
-      <c r="H31" s="7">
+      <c r="H31" s="6">
         <v>339039.0</v>
       </c>
-      <c r="I31" s="7" t="s">
-        <v>106</v>
-      </c>
-      <c r="J31" s="13">
+      <c r="I31" s="6" t="s">
+        <v>110</v>
+      </c>
+      <c r="J31" s="11">
         <v>18462.36</v>
       </c>
-      <c r="K31" s="7">
+      <c r="K31" s="6">
         <v>0.0</v>
       </c>
-      <c r="L31" s="13">
+      <c r="L31" s="11">
         <v>18462.36</v>
       </c>
       <c r="AB31" s="2"/>
@@ -9364,40 +9364,40 @@
       <c r="AH31" s="2"/>
     </row>
     <row r="32">
-      <c r="A32" s="7" t="s">
-        <v>138</v>
-      </c>
-      <c r="B32" s="7" t="s">
-        <v>134</v>
-      </c>
-      <c r="C32" s="13" t="s">
-        <v>139</v>
-      </c>
-      <c r="D32" s="7" t="s">
+      <c r="A32" s="6" t="s">
+        <v>150</v>
+      </c>
+      <c r="B32" s="6" t="s">
+        <v>147</v>
+      </c>
+      <c r="C32" s="11" t="s">
+        <v>152</v>
+      </c>
+      <c r="D32" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="E32" s="11">
+      <c r="E32" s="9">
         <v>46213.0</v>
       </c>
-      <c r="F32" s="7" t="s">
+      <c r="F32" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="G32" s="7">
+      <c r="G32" s="6">
         <v>12.0</v>
       </c>
-      <c r="H32" s="7">
+      <c r="H32" s="6">
         <v>339039.0</v>
       </c>
-      <c r="I32" s="7" t="s">
-        <v>106</v>
-      </c>
-      <c r="J32" s="13">
+      <c r="I32" s="6" t="s">
+        <v>110</v>
+      </c>
+      <c r="J32" s="11">
         <v>1530656.62</v>
       </c>
-      <c r="K32" s="7">
+      <c r="K32" s="6">
         <v>0.0</v>
       </c>
-      <c r="L32" s="13">
+      <c r="L32" s="11">
         <v>1530656.62</v>
       </c>
       <c r="AB32" s="2"/>
@@ -9409,40 +9409,40 @@
       <c r="AH32" s="2"/>
     </row>
     <row r="33">
-      <c r="A33" s="7" t="s">
-        <v>141</v>
-      </c>
-      <c r="B33" s="7" t="s">
-        <v>127</v>
-      </c>
-      <c r="C33" s="13" t="s">
-        <v>143</v>
-      </c>
-      <c r="D33" s="7" t="s">
+      <c r="A33" s="6" t="s">
+        <v>154</v>
+      </c>
+      <c r="B33" s="6" t="s">
+        <v>134</v>
+      </c>
+      <c r="C33" s="11" t="s">
+        <v>156</v>
+      </c>
+      <c r="D33" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="E33" s="11">
+      <c r="E33" s="9">
         <v>46227.0</v>
       </c>
-      <c r="F33" s="7" t="s">
+      <c r="F33" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="G33" s="7">
+      <c r="G33" s="6">
         <v>12.0</v>
       </c>
-      <c r="H33" s="7">
+      <c r="H33" s="6">
         <v>339039.0</v>
       </c>
-      <c r="I33" s="7">
+      <c r="I33" s="6">
         <v>2048.0</v>
       </c>
-      <c r="J33" s="13">
+      <c r="J33" s="11">
         <v>173846.38</v>
       </c>
-      <c r="K33" s="7">
+      <c r="K33" s="6">
         <v>0.0</v>
       </c>
-      <c r="L33" s="13">
+      <c r="L33" s="11">
         <v>173846.38</v>
       </c>
       <c r="AB33" s="2"/>
@@ -9454,40 +9454,40 @@
       <c r="AH33" s="2"/>
     </row>
     <row r="34">
-      <c r="A34" s="7" t="s">
-        <v>146</v>
-      </c>
-      <c r="B34" s="7" t="s">
-        <v>147</v>
-      </c>
-      <c r="C34" s="7" t="s">
-        <v>148</v>
-      </c>
-      <c r="D34" s="7" t="s">
+      <c r="A34" s="6" t="s">
+        <v>159</v>
+      </c>
+      <c r="B34" s="6" t="s">
+        <v>160</v>
+      </c>
+      <c r="C34" s="6" t="s">
+        <v>162</v>
+      </c>
+      <c r="D34" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="E34" s="11">
+      <c r="E34" s="9">
         <v>46240.0</v>
       </c>
-      <c r="F34" s="7" t="s">
+      <c r="F34" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="G34" s="7">
+      <c r="G34" s="6">
         <v>12.0</v>
       </c>
-      <c r="H34" s="7">
+      <c r="H34" s="6">
         <v>339039.0</v>
       </c>
-      <c r="I34" s="7" t="s">
-        <v>150</v>
-      </c>
-      <c r="J34" s="13">
+      <c r="I34" s="6" t="s">
+        <v>164</v>
+      </c>
+      <c r="J34" s="11">
         <v>236343.68</v>
       </c>
-      <c r="K34" s="7">
+      <c r="K34" s="6">
         <v>0.0</v>
       </c>
-      <c r="L34" s="13">
+      <c r="L34" s="11">
         <v>236343.68</v>
       </c>
       <c r="AB34" s="2"/>

</xml_diff>

<commit_message>
Atualização automática: pagamentos (21/09/2026 13:59)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/01_Bases_Originais/005_CELOG_2025/005_CELOG-PAMALS_2025 online.xlsx
+++ b/Contrato 005/Dashboard/01_Bases_Originais/005_CELOG_2025/005_CELOG-PAMALS_2025 online.xlsx
@@ -36,6 +36,9 @@
     <t>2025NE000005</t>
   </si>
   <si>
+    <t>Controle de pagamentos</t>
+  </si>
+  <si>
     <t>C25375</t>
   </si>
   <si>
@@ -45,9 +48,6 @@
     <t>S</t>
   </si>
   <si>
-    <t>Controle de pagamentos</t>
-  </si>
-  <si>
     <t>2025NE000367</t>
   </si>
   <si>
@@ -66,72 +66,72 @@
     <t>25E0387</t>
   </si>
   <si>
+    <t>Número Contrato</t>
+  </si>
+  <si>
     <t>2025NE000371</t>
   </si>
   <si>
     <t>25E0389</t>
   </si>
   <si>
+    <t>UG Executora</t>
+  </si>
+  <si>
+    <t>UG Responsável</t>
+  </si>
+  <si>
     <t>2025NE000413</t>
   </si>
   <si>
+    <t>UG Fiscalizadora</t>
+  </si>
+  <si>
     <t>C25501</t>
   </si>
   <si>
     <t>25E0403</t>
   </si>
   <si>
+    <t>Prazo Final de Execução</t>
+  </si>
+  <si>
+    <t>Prazo Final de Vigência</t>
+  </si>
+  <si>
     <t>20SP</t>
   </si>
   <si>
-    <t>Número Contrato</t>
-  </si>
-  <si>
-    <t>UG Executora</t>
-  </si>
-  <si>
-    <t>UG Responsável</t>
+    <t>Status</t>
+  </si>
+  <si>
+    <t>Ação</t>
+  </si>
+  <si>
+    <t>PAG</t>
   </si>
   <si>
     <t>2025NE000414</t>
   </si>
   <si>
-    <t>UG Fiscalizadora</t>
-  </si>
-  <si>
     <t>C25525</t>
   </si>
   <si>
     <t>25E0431</t>
   </si>
   <si>
-    <t>Prazo Final de Execução</t>
+    <t>Moeda</t>
+  </si>
+  <si>
+    <t>Valor Total do Contrato</t>
+  </si>
+  <si>
+    <t>Valor a Empenhar</t>
   </si>
   <si>
     <t>21EM</t>
   </si>
   <si>
-    <t>Prazo Final de Vigência</t>
-  </si>
-  <si>
-    <t>Status</t>
-  </si>
-  <si>
-    <t>Ação</t>
-  </si>
-  <si>
-    <t>PAG</t>
-  </si>
-  <si>
-    <t>Moeda</t>
-  </si>
-  <si>
-    <t>Valor Total do Contrato</t>
-  </si>
-  <si>
-    <t>Valor a Empenhar</t>
-  </si>
-  <si>
     <t>Valor Empenhado</t>
   </si>
   <si>
@@ -147,42 +147,42 @@
     <t>Tipo Despesa /Receita</t>
   </si>
   <si>
+    <t>Abrir</t>
+  </si>
+  <si>
+    <t>Editar</t>
+  </si>
+  <si>
     <t>2025NE000559</t>
   </si>
   <si>
-    <t>Abrir</t>
-  </si>
-  <si>
     <t>C25545</t>
   </si>
   <si>
-    <t>Editar</t>
-  </si>
-  <si>
     <t>25E0524</t>
   </si>
   <si>
+    <t>005/CELOG-PAMALS/2025</t>
+  </si>
+  <si>
+    <t>CELOG</t>
+  </si>
+  <si>
     <t>20X7</t>
   </si>
   <si>
-    <t>005/CELOG-PAMALS/2025</t>
-  </si>
-  <si>
-    <t>CELOG</t>
-  </si>
-  <si>
     <t>PAMALS</t>
   </si>
   <si>
     <t>2025NE000770</t>
   </si>
   <si>
+    <t>Vigente</t>
+  </si>
+  <si>
     <t>25E0731</t>
   </si>
   <si>
-    <t>Vigente</t>
-  </si>
-  <si>
     <t>2048 20YJ 21EM 219C 20SP 20X7 2000</t>
   </si>
   <si>
@@ -195,12 +195,12 @@
     <t>2025NE000774</t>
   </si>
   <si>
+    <t>VEE ONE-MANUTENCAO E SERVICOS TECNICOS LTDA</t>
+  </si>
+  <si>
     <t>25E0737</t>
   </si>
   <si>
-    <t>VEE ONE-MANUTENCAO E SERVICOS TECNICOS LTDA</t>
-  </si>
-  <si>
     <t>2025NE000843</t>
   </si>
   <si>
@@ -240,18 +240,18 @@
     <t>Módulo</t>
   </si>
   <si>
+    <t>2025NE001627</t>
+  </si>
+  <si>
     <t>Referência</t>
   </si>
   <si>
-    <t>2025NE001627</t>
+    <t>25E1475</t>
   </si>
   <si>
     <t>Nº recibo</t>
   </si>
   <si>
-    <t>25E1475</t>
-  </si>
-  <si>
     <t>Nº</t>
   </si>
   <si>
@@ -303,15 +303,15 @@
     <t>FEV/25</t>
   </si>
   <si>
+    <t>2025NE001689</t>
+  </si>
+  <si>
+    <t>25E1537</t>
+  </si>
+  <si>
     <t>-</t>
   </si>
   <si>
-    <t>2025NE001689</t>
-  </si>
-  <si>
-    <t>25E1537</t>
-  </si>
-  <si>
     <t>2025NE001690</t>
   </si>
   <si>
@@ -330,6 +330,9 @@
     <t>25E1666</t>
   </si>
   <si>
+    <t>2025NP001980</t>
+  </si>
+  <si>
     <t>2025NE001828</t>
   </si>
   <si>
@@ -339,9 +342,6 @@
     <t>25E1667</t>
   </si>
   <si>
-    <t>2025NP001980</t>
-  </si>
-  <si>
     <t>20YJ</t>
   </si>
   <si>
@@ -423,12 +423,12 @@
     <t>2025NE000367, 2025NE000369, 2025NE000371, 2025NE000413</t>
   </si>
   <si>
+    <t>2025NP001979</t>
+  </si>
+  <si>
     <t>2026NE000944</t>
   </si>
   <si>
-    <t>2025NP001979</t>
-  </si>
-  <si>
     <t>26E0906</t>
   </si>
   <si>
@@ -438,28 +438,28 @@
     <t>C26363</t>
   </si>
   <si>
+    <t>ABR/25</t>
+  </si>
+  <si>
     <t>26E0959</t>
   </si>
   <si>
+    <t>2025NE000413, 2025NE000414, 2025NE000559</t>
+  </si>
+  <si>
+    <t>2025NP002341</t>
+  </si>
+  <si>
     <t>20XV</t>
   </si>
   <si>
     <t>2026NE901182</t>
   </si>
   <si>
+    <t>MAI/25</t>
+  </si>
+  <si>
     <t>26E1182</t>
-  </si>
-  <si>
-    <t>ABR/25</t>
-  </si>
-  <si>
-    <t>2025NE000413, 2025NE000414, 2025NE000559</t>
-  </si>
-  <si>
-    <t>2025NP002341</t>
-  </si>
-  <si>
-    <t>MAI/25</t>
   </si>
   <si>
     <t>2025NP002884</t>
@@ -903,33 +903,33 @@
     <xf borderId="0" fillId="0" fontId="2" numFmtId="164" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
       <alignment readingOrder="0"/>
     </xf>
+    <xf borderId="0" fillId="4" fontId="2" numFmtId="0" xfId="0" applyFill="1" applyFont="1"/>
     <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
-    <xf borderId="0" fillId="4" fontId="2" numFmtId="0" xfId="0" applyFill="1" applyFont="1"/>
+    <xf borderId="0" fillId="2" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0" vertical="center"/>
+    </xf>
     <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="2" numFmtId="11" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
-    <xf borderId="0" fillId="2" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
+    <xf borderId="0" fillId="5" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" vertical="center"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="2" numFmtId="164" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" readingOrder="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="4" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
-      <alignment horizontal="center" readingOrder="0"/>
-    </xf>
-    <xf borderId="0" fillId="5" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0" vertical="center"/>
     </xf>
     <xf borderId="0" fillId="4" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
       <alignment vertical="center"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment vertical="center"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="4" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
+      <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
@@ -1449,22 +1449,22 @@
       <c r="S1" s="1"/>
       <c r="T1" s="1"/>
       <c r="U1" s="1"/>
-      <c r="V1" s="5"/>
+      <c r="V1" s="4"/>
     </row>
     <row r="2" ht="59.25" customHeight="1">
-      <c r="A2" s="8"/>
-      <c r="B2" s="11" t="s">
-        <v>5</v>
-      </c>
-      <c r="V2" s="12"/>
-      <c r="W2" s="13"/>
-      <c r="X2" s="13"/>
-      <c r="Y2" s="13"/>
-      <c r="Z2" s="13"/>
-      <c r="AA2" s="13"/>
-      <c r="AB2" s="13"/>
-      <c r="AC2" s="13"/>
-      <c r="AD2" s="13"/>
+      <c r="A2" s="6"/>
+      <c r="B2" s="9" t="s">
+        <v>2</v>
+      </c>
+      <c r="V2" s="11"/>
+      <c r="W2" s="12"/>
+      <c r="X2" s="12"/>
+      <c r="Y2" s="12"/>
+      <c r="Z2" s="12"/>
+      <c r="AA2" s="12"/>
+      <c r="AB2" s="12"/>
+      <c r="AC2" s="12"/>
+      <c r="AD2" s="12"/>
     </row>
     <row r="3" ht="12.75" customHeight="1">
       <c r="A3" s="1"/>
@@ -1488,46 +1488,46 @@
       <c r="S3" s="14"/>
       <c r="T3" s="14"/>
       <c r="U3" s="14"/>
-      <c r="V3" s="5"/>
+      <c r="V3" s="4"/>
     </row>
     <row r="4" ht="12.75" customHeight="1">
       <c r="A4" s="15"/>
       <c r="B4" s="15"/>
       <c r="C4" s="16" t="s">
+        <v>12</v>
+      </c>
+      <c r="D4" s="16" t="s">
+        <v>15</v>
+      </c>
+      <c r="E4" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="F4" s="16" t="s">
         <v>18</v>
       </c>
-      <c r="D4" s="16" t="s">
-        <v>19</v>
-      </c>
-      <c r="E4" s="16" t="s">
-        <v>20</v>
-      </c>
-      <c r="F4" s="16" t="s">
+      <c r="G4" s="17" t="s">
+        <v>21</v>
+      </c>
+      <c r="H4" s="17" t="s">
         <v>22</v>
       </c>
-      <c r="G4" s="17" t="s">
+      <c r="I4" s="16" t="s">
+        <v>24</v>
+      </c>
+      <c r="J4" s="16" t="s">
         <v>25</v>
       </c>
-      <c r="H4" s="17" t="s">
-        <v>27</v>
-      </c>
-      <c r="I4" s="16" t="s">
-        <v>28</v>
-      </c>
-      <c r="J4" s="16" t="s">
-        <v>29</v>
-      </c>
       <c r="K4" s="16" t="s">
+        <v>26</v>
+      </c>
+      <c r="L4" s="16" t="s">
         <v>30</v>
       </c>
-      <c r="L4" s="16" t="s">
+      <c r="M4" s="17" t="s">
         <v>31</v>
       </c>
-      <c r="M4" s="17" t="s">
+      <c r="N4" s="17" t="s">
         <v>32</v>
-      </c>
-      <c r="N4" s="17" t="s">
-        <v>33</v>
       </c>
       <c r="O4" s="17" t="s">
         <v>34</v>
@@ -1545,22 +1545,22 @@
         <v>38</v>
       </c>
       <c r="T4" s="16" t="s">
+        <v>39</v>
+      </c>
+      <c r="U4" s="16" t="s">
         <v>40</v>
       </c>
-      <c r="U4" s="16" t="s">
-        <v>42</v>
-      </c>
-      <c r="V4" s="5"/>
+      <c r="V4" s="4"/>
     </row>
     <row r="5" ht="12.75" customHeight="1">
       <c r="A5" s="15"/>
       <c r="B5" s="15"/>
       <c r="C5" s="19"/>
       <c r="D5" s="20" t="s">
+        <v>44</v>
+      </c>
+      <c r="E5" s="20" t="s">
         <v>45</v>
-      </c>
-      <c r="E5" s="20" t="s">
-        <v>46</v>
       </c>
       <c r="F5" s="20" t="s">
         <v>47</v>
@@ -1575,7 +1575,7 @@
         <v>1564.0</v>
       </c>
       <c r="J5" s="20" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="K5" s="20" t="s">
         <v>51</v>
@@ -1602,15 +1602,15 @@
         <v>1.085943044E7</v>
       </c>
       <c r="S5" s="20" t="s">
-        <v>56</v>
-      </c>
-      <c r="V5" s="5"/>
+        <v>55</v>
+      </c>
+      <c r="V5" s="4"/>
     </row>
     <row r="6" ht="12.75" customHeight="1">
       <c r="A6" s="15"/>
       <c r="B6" s="15"/>
       <c r="L6" s="23"/>
-      <c r="V6" s="5"/>
+      <c r="V6" s="4"/>
     </row>
     <row r="7" ht="12.75" customHeight="1">
       <c r="A7" s="24"/>
@@ -1629,7 +1629,7 @@
       <c r="N7" s="26"/>
       <c r="O7" s="26"/>
       <c r="P7" s="29"/>
-      <c r="V7" s="5"/>
+      <c r="V7" s="4"/>
     </row>
     <row r="8" ht="12.75" customHeight="1">
       <c r="A8" s="24"/>
@@ -1638,10 +1638,10 @@
         <v>69</v>
       </c>
       <c r="D8" s="30" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E8" s="31" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="F8" s="30" t="s">
         <v>74</v>
@@ -1672,7 +1672,7 @@
       </c>
       <c r="O8" s="30"/>
       <c r="P8" s="29"/>
-      <c r="V8" s="5"/>
+      <c r="V8" s="4"/>
     </row>
     <row r="9" ht="19.5" customHeight="1">
       <c r="A9" s="24"/>
@@ -1684,7 +1684,7 @@
         <v>90</v>
       </c>
       <c r="E9" s="35" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="F9" s="36">
         <v>594.0</v>
@@ -1703,7 +1703,7 @@
         <v>748504.24</v>
       </c>
       <c r="L9" s="36" t="s">
-        <v>103</v>
+        <v>100</v>
       </c>
       <c r="M9" s="40">
         <f t="shared" ref="M9:M10" si="1">K9</f>
@@ -1712,7 +1712,7 @@
       <c r="N9" s="41"/>
       <c r="O9" s="26"/>
       <c r="P9" s="29"/>
-      <c r="V9" s="5"/>
+      <c r="V9" s="4"/>
     </row>
     <row r="10" ht="51.0" customHeight="1">
       <c r="A10" s="24"/>
@@ -1722,7 +1722,7 @@
         <v>127</v>
       </c>
       <c r="E10" s="35" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="F10" s="36">
         <v>620.0</v>
@@ -1741,7 +1741,7 @@
         <v>1110378.24</v>
       </c>
       <c r="L10" s="36" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="M10" s="40">
         <f t="shared" si="1"/>
@@ -1750,17 +1750,17 @@
       <c r="N10" s="43"/>
       <c r="O10" s="26"/>
       <c r="P10" s="29"/>
-      <c r="V10" s="5"/>
+      <c r="V10" s="4"/>
     </row>
     <row r="11" ht="12.75" customHeight="1">
       <c r="A11" s="24"/>
       <c r="B11" s="24"/>
       <c r="C11" s="42"/>
       <c r="D11" s="34" t="s">
-        <v>140</v>
+        <v>136</v>
       </c>
       <c r="E11" s="35" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="F11" s="36">
         <v>634.0</v>
@@ -1769,7 +1769,7 @@
         <v>45799.0</v>
       </c>
       <c r="H11" s="36" t="s">
-        <v>141</v>
+        <v>138</v>
       </c>
       <c r="I11" s="37"/>
       <c r="J11" s="37">
@@ -1779,7 +1779,7 @@
         <v>974557.12</v>
       </c>
       <c r="L11" s="35" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
       <c r="M11" s="40">
         <v>974557.12</v>
@@ -1787,17 +1787,17 @@
       <c r="N11" s="43"/>
       <c r="O11" s="26"/>
       <c r="P11" s="29"/>
-      <c r="V11" s="5"/>
+      <c r="V11" s="4"/>
     </row>
     <row r="12" ht="27.75" customHeight="1">
       <c r="A12" s="24"/>
       <c r="B12" s="24"/>
       <c r="C12" s="42"/>
       <c r="D12" s="34" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="E12" s="35" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="F12" s="35">
         <v>660.0</v>
@@ -1824,7 +1824,7 @@
       <c r="N12" s="48"/>
       <c r="O12" s="26"/>
       <c r="P12" s="29"/>
-      <c r="V12" s="5"/>
+      <c r="V12" s="4"/>
     </row>
     <row r="13">
       <c r="A13" s="24"/>
@@ -1834,7 +1834,7 @@
         <v>145</v>
       </c>
       <c r="E13" s="35" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="F13" s="36">
         <v>661.0</v>
@@ -1861,7 +1861,7 @@
       <c r="N13" s="48"/>
       <c r="O13" s="26"/>
       <c r="P13" s="50"/>
-      <c r="V13" s="5"/>
+      <c r="V13" s="4"/>
     </row>
     <row r="14">
       <c r="A14" s="24"/>
@@ -1871,7 +1871,7 @@
         <v>148</v>
       </c>
       <c r="E14" s="35" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="F14" s="35">
         <v>688.0</v>
@@ -1898,7 +1898,7 @@
       <c r="N14" s="43"/>
       <c r="O14" s="26"/>
       <c r="P14" s="29"/>
-      <c r="V14" s="5"/>
+      <c r="V14" s="4"/>
     </row>
     <row r="15">
       <c r="A15" s="24"/>
@@ -1908,7 +1908,7 @@
         <v>151</v>
       </c>
       <c r="E15" s="35" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="F15" s="35">
         <v>696.0</v>
@@ -1934,7 +1934,7 @@
       </c>
       <c r="N15" s="48"/>
       <c r="O15" s="26"/>
-      <c r="V15" s="5"/>
+      <c r="V15" s="4"/>
     </row>
     <row r="16">
       <c r="A16" s="24"/>
@@ -1944,7 +1944,7 @@
         <v>153</v>
       </c>
       <c r="E16" s="35" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="F16" s="35">
         <v>704.0</v>
@@ -1970,7 +1970,7 @@
       </c>
       <c r="N16" s="43"/>
       <c r="O16" s="26"/>
-      <c r="V16" s="5"/>
+      <c r="V16" s="4"/>
     </row>
     <row r="17">
       <c r="A17" s="24"/>
@@ -2004,7 +2004,7 @@
       </c>
       <c r="N17" s="51"/>
       <c r="O17" s="26"/>
-      <c r="V17" s="5"/>
+      <c r="V17" s="4"/>
     </row>
     <row r="18">
       <c r="A18" s="24"/>
@@ -2014,7 +2014,7 @@
         <v>159</v>
       </c>
       <c r="E18" s="35" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="F18" s="35">
         <v>728.0</v>
@@ -2054,7 +2054,7 @@
         <v>162</v>
       </c>
       <c r="E19" s="35" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="F19" s="35">
         <v>278.0</v>
@@ -2417,10 +2417,10 @@
         <v>69</v>
       </c>
       <c r="D29" s="30" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E29" s="31" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="F29" s="31" t="s">
         <v>74</v>
@@ -2475,7 +2475,7 @@
         <v>45791.0</v>
       </c>
       <c r="H30" s="36" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="I30" s="37"/>
       <c r="J30" s="37">
@@ -2818,7 +2818,7 @@
         <v>45968.0</v>
       </c>
       <c r="H37" s="35" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="I37" s="64"/>
       <c r="J37" s="64">
@@ -3127,7 +3127,7 @@
         <v>58868.35</v>
       </c>
       <c r="N44" s="51"/>
-      <c r="V44" s="5"/>
+      <c r="V44" s="4"/>
     </row>
     <row r="45" ht="12.75" customHeight="1">
       <c r="A45" s="15"/>
@@ -3135,7 +3135,7 @@
       <c r="C45" s="42"/>
       <c r="K45" s="74"/>
       <c r="M45" s="74"/>
-      <c r="V45" s="5"/>
+      <c r="V45" s="4"/>
     </row>
     <row r="46" ht="12.75" customHeight="1">
       <c r="A46" s="15"/>
@@ -3143,31 +3143,31 @@
       <c r="C46" s="42"/>
       <c r="K46" s="74"/>
       <c r="M46" s="74"/>
-      <c r="V46" s="5"/>
+      <c r="V46" s="4"/>
     </row>
     <row r="47" ht="12.75" customHeight="1">
       <c r="A47" s="15"/>
       <c r="B47" s="15"/>
       <c r="C47" s="42"/>
-      <c r="V47" s="5"/>
+      <c r="V47" s="4"/>
     </row>
     <row r="48" ht="12.75" customHeight="1">
       <c r="A48" s="15"/>
       <c r="B48" s="15"/>
       <c r="C48" s="42"/>
-      <c r="V48" s="5"/>
+      <c r="V48" s="4"/>
     </row>
     <row r="49" ht="12.75" customHeight="1">
       <c r="A49" s="15"/>
       <c r="B49" s="15"/>
       <c r="C49" s="42"/>
-      <c r="V49" s="5"/>
+      <c r="V49" s="4"/>
     </row>
     <row r="50" ht="12.75" customHeight="1">
       <c r="A50" s="15"/>
       <c r="B50" s="15"/>
       <c r="C50" s="42"/>
-      <c r="V50" s="5"/>
+      <c r="V50" s="4"/>
     </row>
     <row r="51" ht="12.75" customHeight="1">
       <c r="A51" s="15"/>
@@ -3175,7 +3175,7 @@
       <c r="C51" s="55"/>
       <c r="K51" s="74"/>
       <c r="M51" s="74"/>
-      <c r="V51" s="5"/>
+      <c r="V51" s="4"/>
     </row>
     <row r="52" ht="12.75" customHeight="1">
       <c r="A52" s="15"/>
@@ -3199,7 +3199,7 @@
       <c r="S52" s="75"/>
       <c r="T52" s="75"/>
       <c r="U52" s="75"/>
-      <c r="V52" s="5"/>
+      <c r="V52" s="4"/>
     </row>
     <row r="53" ht="12.75" customHeight="1">
       <c r="A53" s="15"/>
@@ -8083,7 +8083,7 @@
       <c r="A2" s="3">
         <v>46258.0</v>
       </c>
-      <c r="L2" s="4" t="s">
+      <c r="L2" s="5" t="s">
         <v>0</v>
       </c>
       <c r="AB2" s="2"/>
@@ -8095,40 +8095,40 @@
       <c r="AH2" s="2"/>
     </row>
     <row r="3">
-      <c r="A3" s="6" t="s">
+      <c r="A3" s="7" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="6" t="s">
-        <v>2</v>
-      </c>
-      <c r="C3" s="7">
+      <c r="B3" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="C3" s="8">
         <v>2.5E32</v>
       </c>
-      <c r="D3" s="6" t="s">
-        <v>3</v>
-      </c>
-      <c r="E3" s="9">
+      <c r="D3" s="7" t="s">
+        <v>4</v>
+      </c>
+      <c r="E3" s="10">
         <v>45686.0</v>
       </c>
-      <c r="F3" s="6" t="s">
-        <v>4</v>
-      </c>
-      <c r="G3" s="6">
+      <c r="F3" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="G3" s="7">
         <v>12.0</v>
       </c>
-      <c r="H3" s="6">
+      <c r="H3" s="7">
         <v>339039.0</v>
       </c>
-      <c r="I3" s="6">
+      <c r="I3" s="7">
         <v>2048.0</v>
       </c>
-      <c r="J3" s="10">
+      <c r="J3" s="13">
         <v>1000.0</v>
       </c>
-      <c r="K3" s="10">
+      <c r="K3" s="13">
         <v>1000.0</v>
       </c>
-      <c r="L3" s="6">
+      <c r="L3" s="7">
         <v>0.0</v>
       </c>
       <c r="AB3" s="2"/>
@@ -8140,40 +8140,40 @@
       <c r="AH3" s="2"/>
     </row>
     <row r="4">
-      <c r="A4" s="6" t="s">
+      <c r="A4" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="B4" s="6" t="s">
+      <c r="B4" s="7" t="s">
         <v>7</v>
       </c>
-      <c r="C4" s="6" t="s">
+      <c r="C4" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="D4" s="6" t="s">
-        <v>3</v>
-      </c>
-      <c r="E4" s="9">
+      <c r="D4" s="7" t="s">
+        <v>4</v>
+      </c>
+      <c r="E4" s="10">
         <v>45762.0</v>
       </c>
-      <c r="F4" s="6" t="s">
-        <v>4</v>
-      </c>
-      <c r="G4" s="6">
+      <c r="F4" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="G4" s="7">
         <v>12.0</v>
       </c>
-      <c r="H4" s="6">
+      <c r="H4" s="7">
         <v>339039.0</v>
       </c>
-      <c r="I4" s="6">
+      <c r="I4" s="7">
         <v>2048.0</v>
       </c>
-      <c r="J4" s="10">
+      <c r="J4" s="13">
         <v>52250.04</v>
       </c>
-      <c r="K4" s="10">
+      <c r="K4" s="13">
         <v>52250.04</v>
       </c>
-      <c r="L4" s="6">
+      <c r="L4" s="7">
         <v>0.0</v>
       </c>
       <c r="AB4" s="2"/>
@@ -8185,40 +8185,40 @@
       <c r="AH4" s="2"/>
     </row>
     <row r="5">
-      <c r="A5" s="6" t="s">
+      <c r="A5" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="B5" s="6" t="s">
+      <c r="B5" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="C5" s="6" t="s">
+      <c r="C5" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="D5" s="6" t="s">
-        <v>3</v>
-      </c>
-      <c r="E5" s="9">
+      <c r="D5" s="7" t="s">
+        <v>4</v>
+      </c>
+      <c r="E5" s="10">
         <v>45762.0</v>
       </c>
-      <c r="F5" s="6" t="s">
-        <v>4</v>
-      </c>
-      <c r="G5" s="6">
+      <c r="F5" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="G5" s="7">
         <v>12.0</v>
       </c>
-      <c r="H5" s="6">
+      <c r="H5" s="7">
         <v>339039.0</v>
       </c>
-      <c r="I5" s="6">
+      <c r="I5" s="7">
         <v>2048.0</v>
       </c>
-      <c r="J5" s="10">
+      <c r="J5" s="13">
         <v>881914.18</v>
       </c>
-      <c r="K5" s="10">
+      <c r="K5" s="13">
         <v>881914.18</v>
       </c>
-      <c r="L5" s="6">
+      <c r="L5" s="7">
         <v>0.0</v>
       </c>
       <c r="AB5" s="2"/>
@@ -8230,40 +8230,40 @@
       <c r="AH5" s="2"/>
     </row>
     <row r="6">
-      <c r="A6" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="B6" s="6" t="s">
+      <c r="A6" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="B6" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="C6" s="6" t="s">
-        <v>13</v>
-      </c>
-      <c r="D6" s="6" t="s">
-        <v>3</v>
-      </c>
-      <c r="E6" s="9">
+      <c r="C6" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="D6" s="7" t="s">
+        <v>4</v>
+      </c>
+      <c r="E6" s="10">
         <v>45762.0</v>
       </c>
-      <c r="F6" s="6" t="s">
-        <v>4</v>
-      </c>
-      <c r="G6" s="6">
+      <c r="F6" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="G6" s="7">
         <v>12.0</v>
       </c>
-      <c r="H6" s="6">
+      <c r="H6" s="7">
         <v>339039.0</v>
       </c>
-      <c r="I6" s="6">
+      <c r="I6" s="7">
         <v>2048.0</v>
       </c>
-      <c r="J6" s="10">
+      <c r="J6" s="13">
         <v>750000.0</v>
       </c>
-      <c r="K6" s="10">
+      <c r="K6" s="13">
         <v>750000.0</v>
       </c>
-      <c r="L6" s="6">
+      <c r="L6" s="7">
         <v>0.0</v>
       </c>
       <c r="AB6" s="2"/>
@@ -8275,40 +8275,40 @@
       <c r="AH6" s="2"/>
     </row>
     <row r="7">
-      <c r="A7" s="6" t="s">
-        <v>14</v>
-      </c>
-      <c r="B7" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="C7" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="D7" s="6" t="s">
-        <v>3</v>
-      </c>
-      <c r="E7" s="9">
+      <c r="A7" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="B7" s="7" t="s">
+        <v>19</v>
+      </c>
+      <c r="C7" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="D7" s="7" t="s">
+        <v>4</v>
+      </c>
+      <c r="E7" s="10">
         <v>45763.0</v>
       </c>
-      <c r="F7" s="6" t="s">
-        <v>4</v>
-      </c>
-      <c r="G7" s="6">
+      <c r="F7" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="G7" s="7">
         <v>12.0</v>
       </c>
-      <c r="H7" s="6">
+      <c r="H7" s="7">
         <v>339039.0</v>
       </c>
-      <c r="I7" s="6" t="s">
-        <v>17</v>
-      </c>
-      <c r="J7" s="10">
+      <c r="I7" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="J7" s="13">
         <v>949835.78</v>
       </c>
-      <c r="K7" s="10">
+      <c r="K7" s="13">
         <v>949835.78</v>
       </c>
-      <c r="L7" s="6">
+      <c r="L7" s="7">
         <v>0.0</v>
       </c>
       <c r="AB7" s="2"/>
@@ -8320,40 +8320,40 @@
       <c r="AH7" s="2"/>
     </row>
     <row r="8">
-      <c r="A8" s="6" t="s">
-        <v>21</v>
-      </c>
-      <c r="B8" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="C8" s="6" t="s">
-        <v>24</v>
-      </c>
-      <c r="D8" s="6" t="s">
-        <v>3</v>
-      </c>
-      <c r="E8" s="9">
+      <c r="A8" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="B8" s="7" t="s">
+        <v>28</v>
+      </c>
+      <c r="C8" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="D8" s="7" t="s">
+        <v>4</v>
+      </c>
+      <c r="E8" s="10">
         <v>45763.0</v>
       </c>
-      <c r="F8" s="6" t="s">
-        <v>4</v>
-      </c>
-      <c r="G8" s="6">
+      <c r="F8" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="G8" s="7">
         <v>12.0</v>
       </c>
-      <c r="H8" s="6">
+      <c r="H8" s="7">
         <v>339039.0</v>
       </c>
-      <c r="I8" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="J8" s="10">
+      <c r="I8" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="J8" s="13">
         <v>524584.95</v>
       </c>
-      <c r="K8" s="10">
+      <c r="K8" s="13">
         <v>524584.95</v>
       </c>
-      <c r="L8" s="6">
+      <c r="L8" s="7">
         <v>0.0</v>
       </c>
       <c r="O8" s="18"/>
@@ -8366,40 +8366,40 @@
       <c r="AH8" s="2"/>
     </row>
     <row r="9">
-      <c r="A9" s="6" t="s">
-        <v>39</v>
-      </c>
-      <c r="B9" s="6" t="s">
+      <c r="A9" s="7" t="s">
         <v>41</v>
       </c>
-      <c r="C9" s="6" t="s">
+      <c r="B9" s="7" t="s">
+        <v>42</v>
+      </c>
+      <c r="C9" s="7" t="s">
         <v>43</v>
       </c>
-      <c r="D9" s="6" t="s">
-        <v>3</v>
-      </c>
-      <c r="E9" s="9">
+      <c r="D9" s="7" t="s">
+        <v>4</v>
+      </c>
+      <c r="E9" s="10">
         <v>45792.0</v>
       </c>
-      <c r="F9" s="6" t="s">
-        <v>4</v>
-      </c>
-      <c r="G9" s="6">
+      <c r="F9" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="G9" s="7">
         <v>12.0</v>
       </c>
-      <c r="H9" s="6">
+      <c r="H9" s="7">
         <v>339039.0</v>
       </c>
-      <c r="I9" s="6" t="s">
-        <v>44</v>
-      </c>
-      <c r="J9" s="10">
+      <c r="I9" s="7" t="s">
+        <v>46</v>
+      </c>
+      <c r="J9" s="13">
         <v>211614.23</v>
       </c>
-      <c r="K9" s="10">
+      <c r="K9" s="13">
         <v>211614.23</v>
       </c>
-      <c r="L9" s="6">
+      <c r="L9" s="7">
         <v>0.0</v>
       </c>
       <c r="AB9" s="2"/>
@@ -8411,40 +8411,40 @@
       <c r="AH9" s="2"/>
     </row>
     <row r="10">
-      <c r="A10" s="6" t="s">
+      <c r="A10" s="7" t="s">
         <v>48</v>
       </c>
-      <c r="B10" s="6" t="s">
+      <c r="B10" s="7" t="s">
         <v>7</v>
       </c>
-      <c r="C10" s="6" t="s">
-        <v>49</v>
-      </c>
-      <c r="D10" s="6" t="s">
-        <v>3</v>
-      </c>
-      <c r="E10" s="9">
+      <c r="C10" s="7" t="s">
+        <v>50</v>
+      </c>
+      <c r="D10" s="7" t="s">
+        <v>4</v>
+      </c>
+      <c r="E10" s="10">
         <v>45825.0</v>
       </c>
-      <c r="F10" s="6" t="s">
-        <v>4</v>
-      </c>
-      <c r="G10" s="6">
+      <c r="F10" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="G10" s="7">
         <v>12.0</v>
       </c>
-      <c r="H10" s="6">
+      <c r="H10" s="7">
         <v>339039.0</v>
       </c>
-      <c r="I10" s="6">
+      <c r="I10" s="7">
         <v>2048.0</v>
       </c>
-      <c r="J10" s="10">
+      <c r="J10" s="13">
         <v>2391157.42</v>
       </c>
-      <c r="K10" s="10">
+      <c r="K10" s="13">
         <v>2391157.41</v>
       </c>
-      <c r="L10" s="10">
+      <c r="L10" s="13">
         <v>0.01</v>
       </c>
       <c r="AB10" s="2"/>
@@ -8456,40 +8456,40 @@
       <c r="AH10" s="2"/>
     </row>
     <row r="11">
-      <c r="A11" s="6" t="s">
+      <c r="A11" s="7" t="s">
         <v>54</v>
       </c>
-      <c r="B11" s="6" t="s">
+      <c r="B11" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="C11" s="6" t="s">
-        <v>55</v>
-      </c>
-      <c r="D11" s="6" t="s">
-        <v>3</v>
-      </c>
-      <c r="E11" s="9">
+      <c r="C11" s="7" t="s">
+        <v>56</v>
+      </c>
+      <c r="D11" s="7" t="s">
+        <v>4</v>
+      </c>
+      <c r="E11" s="10">
         <v>45825.0</v>
       </c>
-      <c r="F11" s="6" t="s">
-        <v>4</v>
-      </c>
-      <c r="G11" s="6">
+      <c r="F11" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="G11" s="7">
         <v>12.0</v>
       </c>
-      <c r="H11" s="6">
+      <c r="H11" s="7">
         <v>339039.0</v>
       </c>
-      <c r="I11" s="6">
+      <c r="I11" s="7">
         <v>2048.0</v>
       </c>
-      <c r="J11" s="10">
+      <c r="J11" s="13">
         <v>618154.39</v>
       </c>
-      <c r="K11" s="10">
+      <c r="K11" s="13">
         <v>618154.38</v>
       </c>
-      <c r="L11" s="6">
+      <c r="L11" s="7">
         <v>0.01</v>
       </c>
       <c r="AB11" s="2"/>
@@ -8501,40 +8501,40 @@
       <c r="AH11" s="2"/>
     </row>
     <row r="12">
-      <c r="A12" s="6" t="s">
+      <c r="A12" s="7" t="s">
         <v>57</v>
       </c>
-      <c r="B12" s="6" t="s">
+      <c r="B12" s="7" t="s">
         <v>58</v>
       </c>
-      <c r="C12" s="6" t="s">
+      <c r="C12" s="7" t="s">
         <v>59</v>
       </c>
-      <c r="D12" s="6" t="s">
-        <v>3</v>
-      </c>
-      <c r="E12" s="9">
+      <c r="D12" s="7" t="s">
+        <v>4</v>
+      </c>
+      <c r="E12" s="10">
         <v>45832.0</v>
       </c>
-      <c r="F12" s="6" t="s">
-        <v>4</v>
-      </c>
-      <c r="G12" s="6">
+      <c r="F12" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="G12" s="7">
         <v>12.0</v>
       </c>
-      <c r="H12" s="6">
+      <c r="H12" s="7">
         <v>339039.0</v>
       </c>
-      <c r="I12" s="6" t="s">
+      <c r="I12" s="7" t="s">
         <v>60</v>
       </c>
-      <c r="J12" s="10">
+      <c r="J12" s="13">
         <v>1600334.09</v>
       </c>
-      <c r="K12" s="10">
+      <c r="K12" s="13">
         <v>1600334.09</v>
       </c>
-      <c r="L12" s="6">
+      <c r="L12" s="7">
         <v>0.0</v>
       </c>
       <c r="AB12" s="2"/>
@@ -8546,40 +8546,40 @@
       <c r="AH12" s="2"/>
     </row>
     <row r="13">
-      <c r="A13" s="6" t="s">
+      <c r="A13" s="7" t="s">
         <v>61</v>
       </c>
-      <c r="B13" s="6" t="s">
+      <c r="B13" s="7" t="s">
         <v>7</v>
       </c>
-      <c r="C13" s="6" t="s">
+      <c r="C13" s="7" t="s">
         <v>62</v>
       </c>
-      <c r="D13" s="6" t="s">
-        <v>3</v>
-      </c>
-      <c r="E13" s="9">
+      <c r="D13" s="7" t="s">
+        <v>4</v>
+      </c>
+      <c r="E13" s="10">
         <v>45863.0</v>
       </c>
-      <c r="F13" s="6" t="s">
-        <v>4</v>
-      </c>
-      <c r="G13" s="6">
+      <c r="F13" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="G13" s="7">
         <v>12.0</v>
       </c>
-      <c r="H13" s="6">
+      <c r="H13" s="7">
         <v>339039.0</v>
       </c>
-      <c r="I13" s="6">
+      <c r="I13" s="7">
         <v>2048.0</v>
       </c>
-      <c r="J13" s="10">
+      <c r="J13" s="13">
         <v>2364771.07</v>
       </c>
-      <c r="K13" s="10">
+      <c r="K13" s="13">
         <v>2364771.06</v>
       </c>
-      <c r="L13" s="10">
+      <c r="L13" s="13">
         <v>0.01</v>
       </c>
       <c r="M13" s="28"/>
@@ -8592,40 +8592,40 @@
       <c r="AH13" s="2"/>
     </row>
     <row r="14">
-      <c r="A14" s="6" t="s">
+      <c r="A14" s="7" t="s">
         <v>63</v>
       </c>
-      <c r="B14" s="6" t="s">
+      <c r="B14" s="7" t="s">
         <v>64</v>
       </c>
-      <c r="C14" s="6" t="s">
+      <c r="C14" s="7" t="s">
         <v>65</v>
       </c>
-      <c r="D14" s="6" t="s">
-        <v>3</v>
-      </c>
-      <c r="E14" s="9">
+      <c r="D14" s="7" t="s">
+        <v>4</v>
+      </c>
+      <c r="E14" s="10">
         <v>45887.0</v>
       </c>
-      <c r="F14" s="6" t="s">
-        <v>4</v>
-      </c>
-      <c r="G14" s="6">
+      <c r="F14" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="G14" s="7">
         <v>12.0</v>
       </c>
-      <c r="H14" s="6">
+      <c r="H14" s="7">
         <v>339039.0</v>
       </c>
-      <c r="I14" s="6" t="s">
-        <v>44</v>
-      </c>
-      <c r="J14" s="10">
+      <c r="I14" s="7" t="s">
+        <v>46</v>
+      </c>
+      <c r="J14" s="13">
         <v>968237.39</v>
       </c>
-      <c r="K14" s="10">
+      <c r="K14" s="13">
         <v>968237.39</v>
       </c>
-      <c r="L14" s="6">
+      <c r="L14" s="7">
         <v>0.0</v>
       </c>
       <c r="AB14" s="2"/>
@@ -8637,40 +8637,40 @@
       <c r="AH14" s="2"/>
     </row>
     <row r="15">
-      <c r="A15" s="6" t="s">
+      <c r="A15" s="7" t="s">
         <v>66</v>
       </c>
-      <c r="B15" s="6" t="s">
+      <c r="B15" s="7" t="s">
         <v>67</v>
       </c>
-      <c r="C15" s="6" t="s">
+      <c r="C15" s="7" t="s">
         <v>68</v>
       </c>
-      <c r="D15" s="6" t="s">
-        <v>3</v>
-      </c>
-      <c r="E15" s="9">
+      <c r="D15" s="7" t="s">
+        <v>4</v>
+      </c>
+      <c r="E15" s="10">
         <v>45924.0</v>
       </c>
-      <c r="F15" s="6" t="s">
-        <v>4</v>
-      </c>
-      <c r="G15" s="6">
+      <c r="F15" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="G15" s="7">
         <v>12.0</v>
       </c>
-      <c r="H15" s="6">
+      <c r="H15" s="7">
         <v>339039.0</v>
       </c>
-      <c r="I15" s="6" t="s">
-        <v>17</v>
-      </c>
-      <c r="J15" s="10">
+      <c r="I15" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="J15" s="13">
         <v>1011677.95</v>
       </c>
-      <c r="K15" s="10">
+      <c r="K15" s="13">
         <v>1011677.95</v>
       </c>
-      <c r="L15" s="6">
+      <c r="L15" s="7">
         <v>0.0</v>
       </c>
       <c r="AB15" s="2"/>
@@ -8682,40 +8682,40 @@
       <c r="AH15" s="2"/>
     </row>
     <row r="16">
-      <c r="A16" s="6" t="s">
-        <v>71</v>
-      </c>
-      <c r="B16" s="6" t="s">
+      <c r="A16" s="7" t="s">
+        <v>70</v>
+      </c>
+      <c r="B16" s="7" t="s">
         <v>7</v>
       </c>
-      <c r="C16" s="6" t="s">
-        <v>73</v>
-      </c>
-      <c r="D16" s="6" t="s">
-        <v>3</v>
-      </c>
-      <c r="E16" s="9">
+      <c r="C16" s="7" t="s">
+        <v>72</v>
+      </c>
+      <c r="D16" s="7" t="s">
+        <v>4</v>
+      </c>
+      <c r="E16" s="10">
         <v>45929.0</v>
       </c>
-      <c r="F16" s="6" t="s">
-        <v>4</v>
-      </c>
-      <c r="G16" s="6">
+      <c r="F16" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="G16" s="7">
         <v>12.0</v>
       </c>
-      <c r="H16" s="6">
+      <c r="H16" s="7">
         <v>339039.0</v>
       </c>
-      <c r="I16" s="6">
+      <c r="I16" s="7">
         <v>2048.0</v>
       </c>
-      <c r="J16" s="10">
+      <c r="J16" s="13">
         <v>1580293.02</v>
       </c>
-      <c r="K16" s="10">
+      <c r="K16" s="13">
         <v>1580293.02</v>
       </c>
-      <c r="L16" s="10">
+      <c r="L16" s="13">
         <v>0.0</v>
       </c>
       <c r="AB16" s="2"/>
@@ -8727,40 +8727,40 @@
       <c r="AH16" s="2"/>
     </row>
     <row r="17">
-      <c r="A17" s="6" t="s">
+      <c r="A17" s="7" t="s">
         <v>81</v>
       </c>
-      <c r="B17" s="6" t="s">
+      <c r="B17" s="7" t="s">
         <v>82</v>
       </c>
-      <c r="C17" s="6" t="s">
+      <c r="C17" s="7" t="s">
         <v>83</v>
       </c>
-      <c r="D17" s="6" t="s">
-        <v>3</v>
-      </c>
-      <c r="E17" s="9">
+      <c r="D17" s="7" t="s">
+        <v>4</v>
+      </c>
+      <c r="E17" s="10">
         <v>45930.0</v>
       </c>
-      <c r="F17" s="6" t="s">
-        <v>4</v>
-      </c>
-      <c r="G17" s="6">
+      <c r="F17" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="G17" s="7">
         <v>12.0</v>
       </c>
-      <c r="H17" s="6">
+      <c r="H17" s="7">
         <v>339039.0</v>
       </c>
-      <c r="I17" s="6">
+      <c r="I17" s="7">
         <v>2048.0</v>
       </c>
-      <c r="J17" s="10">
+      <c r="J17" s="13">
         <v>34065.36</v>
       </c>
-      <c r="K17" s="6">
+      <c r="K17" s="7">
         <v>0.01</v>
       </c>
-      <c r="L17" s="10">
+      <c r="L17" s="13">
         <v>34065.35</v>
       </c>
       <c r="AB17" s="2"/>
@@ -8772,40 +8772,40 @@
       <c r="AH17" s="2"/>
     </row>
     <row r="18">
-      <c r="A18" s="6" t="s">
+      <c r="A18" s="7" t="s">
         <v>86</v>
       </c>
-      <c r="B18" s="6" t="s">
+      <c r="B18" s="7" t="s">
         <v>64</v>
       </c>
-      <c r="C18" s="6" t="s">
+      <c r="C18" s="7" t="s">
         <v>87</v>
       </c>
-      <c r="D18" s="6" t="s">
-        <v>3</v>
-      </c>
-      <c r="E18" s="9">
+      <c r="D18" s="7" t="s">
+        <v>4</v>
+      </c>
+      <c r="E18" s="10">
         <v>45938.0</v>
       </c>
-      <c r="F18" s="6" t="s">
-        <v>4</v>
-      </c>
-      <c r="G18" s="6">
+      <c r="F18" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="G18" s="7">
         <v>12.0</v>
       </c>
-      <c r="H18" s="6">
+      <c r="H18" s="7">
         <v>339039.0</v>
       </c>
-      <c r="I18" s="6" t="s">
-        <v>44</v>
-      </c>
-      <c r="J18" s="10">
+      <c r="I18" s="7" t="s">
+        <v>46</v>
+      </c>
+      <c r="J18" s="13">
         <v>63746.85</v>
       </c>
-      <c r="K18" s="10">
+      <c r="K18" s="13">
         <v>63746.85</v>
       </c>
-      <c r="L18" s="6">
+      <c r="L18" s="7">
         <v>0.0</v>
       </c>
       <c r="AB18" s="2"/>
@@ -8817,40 +8817,40 @@
       <c r="AH18" s="2"/>
     </row>
     <row r="19">
-      <c r="A19" s="6" t="s">
+      <c r="A19" s="7" t="s">
         <v>88</v>
       </c>
-      <c r="B19" s="6" t="s">
+      <c r="B19" s="7" t="s">
         <v>58</v>
       </c>
-      <c r="C19" s="6" t="s">
+      <c r="C19" s="7" t="s">
         <v>89</v>
       </c>
-      <c r="D19" s="6" t="s">
-        <v>3</v>
-      </c>
-      <c r="E19" s="9">
+      <c r="D19" s="7" t="s">
+        <v>4</v>
+      </c>
+      <c r="E19" s="10">
         <v>45938.0</v>
       </c>
-      <c r="F19" s="6" t="s">
-        <v>4</v>
-      </c>
-      <c r="G19" s="6">
+      <c r="F19" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="G19" s="7">
         <v>12.0</v>
       </c>
-      <c r="H19" s="6">
+      <c r="H19" s="7">
         <v>339039.0</v>
       </c>
-      <c r="I19" s="6" t="s">
+      <c r="I19" s="7" t="s">
         <v>60</v>
       </c>
-      <c r="J19" s="10">
+      <c r="J19" s="13">
         <v>947931.1</v>
       </c>
-      <c r="K19" s="10">
+      <c r="K19" s="13">
         <v>947931.1</v>
       </c>
-      <c r="L19" s="6">
+      <c r="L19" s="7">
         <v>0.0</v>
       </c>
       <c r="AB19" s="2"/>
@@ -8862,40 +8862,40 @@
       <c r="AH19" s="2"/>
     </row>
     <row r="20">
-      <c r="A20" s="6" t="s">
+      <c r="A20" s="7" t="s">
+        <v>91</v>
+      </c>
+      <c r="B20" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="C20" s="7" t="s">
         <v>92</v>
       </c>
-      <c r="B20" s="6" t="s">
-        <v>7</v>
-      </c>
-      <c r="C20" s="6" t="s">
-        <v>93</v>
-      </c>
-      <c r="D20" s="6" t="s">
-        <v>3</v>
-      </c>
-      <c r="E20" s="9">
+      <c r="D20" s="7" t="s">
+        <v>4</v>
+      </c>
+      <c r="E20" s="10">
         <v>45938.0</v>
       </c>
-      <c r="F20" s="6" t="s">
-        <v>4</v>
-      </c>
-      <c r="G20" s="6">
+      <c r="F20" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="G20" s="7">
         <v>12.0</v>
       </c>
-      <c r="H20" s="6">
+      <c r="H20" s="7">
         <v>339039.0</v>
       </c>
-      <c r="I20" s="6">
+      <c r="I20" s="7">
         <v>2048.0</v>
       </c>
-      <c r="J20" s="10">
+      <c r="J20" s="13">
         <v>259790.57</v>
       </c>
-      <c r="K20" s="10">
+      <c r="K20" s="13">
         <v>259790.57</v>
       </c>
-      <c r="L20" s="6">
+      <c r="L20" s="7">
         <v>0.0</v>
       </c>
       <c r="AB20" s="2"/>
@@ -8907,40 +8907,40 @@
       <c r="AH20" s="2"/>
     </row>
     <row r="21">
-      <c r="A21" s="6" t="s">
+      <c r="A21" s="7" t="s">
         <v>94</v>
       </c>
-      <c r="B21" s="6" t="s">
+      <c r="B21" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="C21" s="6" t="s">
+      <c r="C21" s="7" t="s">
         <v>95</v>
       </c>
-      <c r="D21" s="6" t="s">
-        <v>3</v>
-      </c>
-      <c r="E21" s="9">
+      <c r="D21" s="7" t="s">
+        <v>4</v>
+      </c>
+      <c r="E21" s="10">
         <v>45938.0</v>
       </c>
-      <c r="F21" s="6" t="s">
-        <v>4</v>
-      </c>
-      <c r="G21" s="6">
+      <c r="F21" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="G21" s="7">
         <v>12.0</v>
       </c>
-      <c r="H21" s="6">
+      <c r="H21" s="7">
         <v>339039.0</v>
       </c>
-      <c r="I21" s="6">
+      <c r="I21" s="7">
         <v>2048.0</v>
       </c>
-      <c r="J21" s="10">
+      <c r="J21" s="13">
         <v>170479.3</v>
       </c>
-      <c r="K21" s="10">
+      <c r="K21" s="13">
         <v>170479.3</v>
       </c>
-      <c r="L21" s="6">
+      <c r="L21" s="7">
         <v>0.0</v>
       </c>
       <c r="AB21" s="2"/>
@@ -8952,40 +8952,40 @@
       <c r="AH21" s="2"/>
     </row>
     <row r="22">
-      <c r="A22" s="6" t="s">
+      <c r="A22" s="7" t="s">
         <v>97</v>
       </c>
-      <c r="B22" s="6" t="s">
+      <c r="B22" s="7" t="s">
         <v>98</v>
       </c>
-      <c r="C22" s="6" t="s">
+      <c r="C22" s="7" t="s">
         <v>99</v>
       </c>
-      <c r="D22" s="6" t="s">
-        <v>3</v>
+      <c r="D22" s="7" t="s">
+        <v>4</v>
       </c>
       <c r="E22" s="38">
         <v>45953.0</v>
       </c>
-      <c r="F22" s="6" t="s">
-        <v>4</v>
-      </c>
-      <c r="G22" s="6">
+      <c r="F22" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="G22" s="7">
         <v>12.0</v>
       </c>
-      <c r="H22" s="6">
+      <c r="H22" s="7">
         <v>339039.0</v>
       </c>
-      <c r="I22" s="6">
+      <c r="I22" s="7">
         <v>2000.0</v>
       </c>
-      <c r="J22" s="10">
+      <c r="J22" s="13">
         <v>1500000.0</v>
       </c>
-      <c r="K22" s="10">
+      <c r="K22" s="13">
         <v>1500000.0</v>
       </c>
-      <c r="L22" s="10">
+      <c r="L22" s="13">
         <v>0.0</v>
       </c>
       <c r="AB22" s="2"/>
@@ -8997,40 +8997,40 @@
       <c r="AH22" s="2"/>
     </row>
     <row r="23">
-      <c r="A23" s="6" t="s">
-        <v>100</v>
-      </c>
-      <c r="B23" s="6" t="s">
+      <c r="A23" s="7" t="s">
         <v>101</v>
       </c>
-      <c r="C23" s="6" t="s">
+      <c r="B23" s="7" t="s">
         <v>102</v>
       </c>
-      <c r="D23" s="6" t="s">
-        <v>3</v>
+      <c r="C23" s="7" t="s">
+        <v>103</v>
+      </c>
+      <c r="D23" s="7" t="s">
+        <v>4</v>
       </c>
       <c r="E23" s="38">
         <v>45953.0</v>
       </c>
-      <c r="F23" s="6" t="s">
-        <v>4</v>
-      </c>
-      <c r="G23" s="6">
+      <c r="F23" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="G23" s="7">
         <v>12.0</v>
       </c>
-      <c r="H23" s="6">
+      <c r="H23" s="7">
         <v>339039.0</v>
       </c>
-      <c r="I23" s="6" t="s">
+      <c r="I23" s="7" t="s">
         <v>104</v>
       </c>
-      <c r="J23" s="10">
+      <c r="J23" s="13">
         <v>1000001.64</v>
       </c>
-      <c r="K23" s="10">
+      <c r="K23" s="13">
         <v>1000001.64</v>
       </c>
-      <c r="L23" s="6">
+      <c r="L23" s="7">
         <v>0.0</v>
       </c>
       <c r="AB23" s="2"/>
@@ -9042,40 +9042,40 @@
       <c r="AH23" s="2"/>
     </row>
     <row r="24">
-      <c r="A24" s="6" t="s">
+      <c r="A24" s="7" t="s">
         <v>105</v>
       </c>
-      <c r="B24" s="6" t="s">
+      <c r="B24" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="C24" s="6" t="s">
+      <c r="C24" s="7" t="s">
         <v>106</v>
       </c>
-      <c r="D24" s="6" t="s">
-        <v>3</v>
+      <c r="D24" s="7" t="s">
+        <v>4</v>
       </c>
       <c r="E24" s="38">
         <v>45953.0</v>
       </c>
-      <c r="F24" s="6" t="s">
-        <v>4</v>
-      </c>
-      <c r="G24" s="6">
+      <c r="F24" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="G24" s="7">
         <v>12.0</v>
       </c>
-      <c r="H24" s="6">
+      <c r="H24" s="7">
         <v>339039.0</v>
       </c>
-      <c r="I24" s="6">
+      <c r="I24" s="7">
         <v>2048.0</v>
       </c>
-      <c r="J24" s="10">
+      <c r="J24" s="13">
         <v>68405.66</v>
       </c>
-      <c r="K24" s="10">
+      <c r="K24" s="13">
         <v>68405.66</v>
       </c>
-      <c r="L24" s="6">
+      <c r="L24" s="7">
         <v>0.0</v>
       </c>
       <c r="AB24" s="2"/>
@@ -9087,40 +9087,40 @@
       <c r="AH24" s="2"/>
     </row>
     <row r="25">
-      <c r="A25" s="6" t="s">
+      <c r="A25" s="7" t="s">
         <v>107</v>
       </c>
-      <c r="B25" s="6" t="s">
+      <c r="B25" s="7" t="s">
         <v>108</v>
       </c>
-      <c r="C25" s="6" t="s">
+      <c r="C25" s="7" t="s">
         <v>109</v>
       </c>
-      <c r="D25" s="6" t="s">
-        <v>3</v>
+      <c r="D25" s="7" t="s">
+        <v>4</v>
       </c>
       <c r="E25" s="38">
         <v>45975.0</v>
       </c>
-      <c r="F25" s="6" t="s">
-        <v>4</v>
-      </c>
-      <c r="G25" s="6">
+      <c r="F25" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="G25" s="7">
         <v>12.0</v>
       </c>
-      <c r="H25" s="6">
+      <c r="H25" s="7">
         <v>339039.0</v>
       </c>
-      <c r="I25" s="6" t="s">
+      <c r="I25" s="7" t="s">
         <v>104</v>
       </c>
-      <c r="J25" s="10">
+      <c r="J25" s="13">
         <v>1157673.06</v>
       </c>
-      <c r="K25" s="10">
+      <c r="K25" s="13">
         <v>1157673.06</v>
       </c>
-      <c r="L25" s="6">
+      <c r="L25" s="7">
         <v>0.0</v>
       </c>
       <c r="AB25" s="2"/>
@@ -9132,40 +9132,40 @@
       <c r="AH25" s="2"/>
     </row>
     <row r="26">
-      <c r="A26" s="6" t="s">
+      <c r="A26" s="7" t="s">
         <v>110</v>
       </c>
-      <c r="B26" s="6" t="s">
+      <c r="B26" s="7" t="s">
         <v>7</v>
       </c>
-      <c r="C26" s="6" t="s">
+      <c r="C26" s="7" t="s">
         <v>111</v>
       </c>
-      <c r="D26" s="6" t="s">
-        <v>3</v>
+      <c r="D26" s="7" t="s">
+        <v>4</v>
       </c>
       <c r="E26" s="38">
         <v>45989.0</v>
       </c>
-      <c r="F26" s="6" t="s">
-        <v>4</v>
-      </c>
-      <c r="G26" s="6">
+      <c r="F26" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="G26" s="7">
         <v>12.0</v>
       </c>
-      <c r="H26" s="6">
+      <c r="H26" s="7">
         <v>339039.0</v>
       </c>
-      <c r="I26" s="6">
+      <c r="I26" s="7">
         <v>2048.0</v>
       </c>
-      <c r="J26" s="10">
+      <c r="J26" s="13">
         <v>34065.36</v>
       </c>
-      <c r="K26" s="10">
+      <c r="K26" s="13">
         <v>34065.36</v>
       </c>
-      <c r="L26" s="6">
+      <c r="L26" s="7">
         <v>0.0</v>
       </c>
       <c r="AB26" s="2"/>
@@ -9177,40 +9177,40 @@
       <c r="AH26" s="2"/>
     </row>
     <row r="27">
-      <c r="A27" s="6" t="s">
+      <c r="A27" s="7" t="s">
         <v>112</v>
       </c>
-      <c r="B27" s="6" t="s">
+      <c r="B27" s="7" t="s">
         <v>113</v>
       </c>
-      <c r="C27" s="6" t="s">
+      <c r="C27" s="7" t="s">
         <v>114</v>
       </c>
-      <c r="D27" s="6" t="s">
-        <v>3</v>
-      </c>
-      <c r="E27" s="9">
+      <c r="D27" s="7" t="s">
+        <v>4</v>
+      </c>
+      <c r="E27" s="10">
         <v>46104.0</v>
       </c>
-      <c r="F27" s="6" t="s">
-        <v>4</v>
-      </c>
-      <c r="G27" s="6">
+      <c r="F27" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="G27" s="7">
         <v>12.0</v>
       </c>
-      <c r="H27" s="6">
+      <c r="H27" s="7">
         <v>339039.0</v>
       </c>
-      <c r="I27" s="6">
+      <c r="I27" s="7">
         <v>2048.0</v>
       </c>
-      <c r="J27" s="10">
+      <c r="J27" s="13">
         <v>1770880.5</v>
       </c>
-      <c r="K27" s="10">
+      <c r="K27" s="13">
         <v>843261.89</v>
       </c>
-      <c r="L27" s="10">
+      <c r="L27" s="13">
         <v>927618.61</v>
       </c>
       <c r="AB27" s="2"/>
@@ -9222,40 +9222,40 @@
       <c r="AH27" s="2"/>
     </row>
     <row r="28">
-      <c r="A28" s="6" t="s">
+      <c r="A28" s="7" t="s">
         <v>115</v>
       </c>
-      <c r="B28" s="6" t="s">
+      <c r="B28" s="7" t="s">
         <v>116</v>
       </c>
-      <c r="C28" s="6" t="s">
+      <c r="C28" s="7" t="s">
         <v>117</v>
       </c>
-      <c r="D28" s="6" t="s">
-        <v>3</v>
-      </c>
-      <c r="E28" s="9">
+      <c r="D28" s="7" t="s">
+        <v>4</v>
+      </c>
+      <c r="E28" s="10">
         <v>46120.0</v>
       </c>
-      <c r="F28" s="6" t="s">
-        <v>4</v>
-      </c>
-      <c r="G28" s="6">
+      <c r="F28" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="G28" s="7">
         <v>12.0</v>
       </c>
-      <c r="H28" s="6">
+      <c r="H28" s="7">
         <v>339039.0</v>
       </c>
-      <c r="I28" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="J28" s="10">
+      <c r="I28" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="J28" s="13">
         <v>1912292.52</v>
       </c>
-      <c r="K28" s="10">
+      <c r="K28" s="13">
         <v>1629834.48</v>
       </c>
-      <c r="L28" s="10">
+      <c r="L28" s="13">
         <v>282458.04</v>
       </c>
       <c r="AB28" s="2"/>
@@ -9267,40 +9267,40 @@
       <c r="AH28" s="2"/>
     </row>
     <row r="29">
-      <c r="A29" s="6" t="s">
+      <c r="A29" s="7" t="s">
         <v>118</v>
       </c>
-      <c r="B29" s="6" t="s">
+      <c r="B29" s="7" t="s">
         <v>119</v>
       </c>
-      <c r="C29" s="6" t="s">
+      <c r="C29" s="7" t="s">
         <v>120</v>
       </c>
-      <c r="D29" s="6" t="s">
-        <v>3</v>
-      </c>
-      <c r="E29" s="9">
+      <c r="D29" s="7" t="s">
+        <v>4</v>
+      </c>
+      <c r="E29" s="10">
         <v>46196.0</v>
       </c>
-      <c r="F29" s="6" t="s">
-        <v>4</v>
-      </c>
-      <c r="G29" s="6">
+      <c r="F29" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="G29" s="7">
         <v>12.0</v>
       </c>
-      <c r="H29" s="6">
+      <c r="H29" s="7">
         <v>339039.0</v>
       </c>
-      <c r="I29" s="6">
+      <c r="I29" s="7">
         <v>2048.0</v>
       </c>
-      <c r="J29" s="10">
+      <c r="J29" s="13">
         <v>1496713.48</v>
       </c>
-      <c r="K29" s="6">
+      <c r="K29" s="7">
         <v>0.0</v>
       </c>
-      <c r="L29" s="10">
+      <c r="L29" s="13">
         <v>1496713.48</v>
       </c>
       <c r="AB29" s="2"/>
@@ -9312,40 +9312,40 @@
       <c r="AH29" s="2"/>
     </row>
     <row r="30">
-      <c r="A30" s="6" t="s">
+      <c r="A30" s="7" t="s">
         <v>121</v>
       </c>
-      <c r="B30" s="6" t="s">
+      <c r="B30" s="7" t="s">
         <v>122</v>
       </c>
-      <c r="C30" s="6" t="s">
+      <c r="C30" s="7" t="s">
         <v>123</v>
       </c>
-      <c r="D30" s="6" t="s">
-        <v>3</v>
-      </c>
-      <c r="E30" s="9">
+      <c r="D30" s="7" t="s">
+        <v>4</v>
+      </c>
+      <c r="E30" s="10">
         <v>46205.0</v>
       </c>
-      <c r="F30" s="6" t="s">
-        <v>4</v>
-      </c>
-      <c r="G30" s="6">
+      <c r="F30" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="G30" s="7">
         <v>12.0</v>
       </c>
-      <c r="H30" s="6">
+      <c r="H30" s="7">
         <v>339039.0</v>
       </c>
-      <c r="I30" s="6" t="s">
-        <v>17</v>
-      </c>
-      <c r="J30" s="10">
+      <c r="I30" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="J30" s="13">
         <v>624166.14</v>
       </c>
-      <c r="K30" s="6">
+      <c r="K30" s="7">
         <v>0.0</v>
       </c>
-      <c r="L30" s="10">
+      <c r="L30" s="13">
         <v>624166.14</v>
       </c>
       <c r="AB30" s="2"/>
@@ -9357,40 +9357,40 @@
       <c r="AH30" s="2"/>
     </row>
     <row r="31">
-      <c r="A31" s="6" t="s">
+      <c r="A31" s="7" t="s">
         <v>124</v>
       </c>
-      <c r="B31" s="6" t="s">
+      <c r="B31" s="7" t="s">
         <v>125</v>
       </c>
-      <c r="C31" s="6" t="s">
+      <c r="C31" s="7" t="s">
         <v>126</v>
       </c>
-      <c r="D31" s="6" t="s">
-        <v>3</v>
-      </c>
-      <c r="E31" s="9">
+      <c r="D31" s="7" t="s">
+        <v>4</v>
+      </c>
+      <c r="E31" s="10">
         <v>46205.0</v>
       </c>
-      <c r="F31" s="6" t="s">
-        <v>4</v>
-      </c>
-      <c r="G31" s="6">
+      <c r="F31" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="G31" s="7">
         <v>12.0</v>
       </c>
-      <c r="H31" s="6">
+      <c r="H31" s="7">
         <v>339039.0</v>
       </c>
-      <c r="I31" s="6" t="s">
+      <c r="I31" s="7" t="s">
         <v>104</v>
       </c>
-      <c r="J31" s="10">
+      <c r="J31" s="13">
         <v>18462.36</v>
       </c>
-      <c r="K31" s="6">
+      <c r="K31" s="7">
         <v>0.0</v>
       </c>
-      <c r="L31" s="10">
+      <c r="L31" s="13">
         <v>18462.36</v>
       </c>
       <c r="AB31" s="2"/>
@@ -9402,40 +9402,40 @@
       <c r="AH31" s="2"/>
     </row>
     <row r="32">
-      <c r="A32" s="6" t="s">
+      <c r="A32" s="7" t="s">
         <v>128</v>
       </c>
-      <c r="B32" s="6" t="s">
+      <c r="B32" s="7" t="s">
         <v>125</v>
       </c>
-      <c r="C32" s="10" t="s">
+      <c r="C32" s="13" t="s">
         <v>129</v>
       </c>
-      <c r="D32" s="6" t="s">
-        <v>3</v>
-      </c>
-      <c r="E32" s="9">
+      <c r="D32" s="7" t="s">
+        <v>4</v>
+      </c>
+      <c r="E32" s="10">
         <v>46213.0</v>
       </c>
-      <c r="F32" s="6" t="s">
-        <v>4</v>
-      </c>
-      <c r="G32" s="6">
+      <c r="F32" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="G32" s="7">
         <v>12.0</v>
       </c>
-      <c r="H32" s="6">
+      <c r="H32" s="7">
         <v>339039.0</v>
       </c>
-      <c r="I32" s="6" t="s">
+      <c r="I32" s="7" t="s">
         <v>104</v>
       </c>
-      <c r="J32" s="10">
+      <c r="J32" s="13">
         <v>1530656.62</v>
       </c>
-      <c r="K32" s="6">
+      <c r="K32" s="7">
         <v>0.0</v>
       </c>
-      <c r="L32" s="10">
+      <c r="L32" s="13">
         <v>1530656.62</v>
       </c>
       <c r="AB32" s="2"/>
@@ -9447,40 +9447,40 @@
       <c r="AH32" s="2"/>
     </row>
     <row r="33">
-      <c r="A33" s="6" t="s">
-        <v>131</v>
-      </c>
-      <c r="B33" s="6" t="s">
+      <c r="A33" s="7" t="s">
+        <v>132</v>
+      </c>
+      <c r="B33" s="7" t="s">
         <v>119</v>
       </c>
-      <c r="C33" s="10" t="s">
+      <c r="C33" s="13" t="s">
         <v>133</v>
       </c>
-      <c r="D33" s="6" t="s">
-        <v>3</v>
-      </c>
-      <c r="E33" s="9">
+      <c r="D33" s="7" t="s">
+        <v>4</v>
+      </c>
+      <c r="E33" s="10">
         <v>46227.0</v>
       </c>
-      <c r="F33" s="6" t="s">
-        <v>4</v>
-      </c>
-      <c r="G33" s="6">
+      <c r="F33" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="G33" s="7">
         <v>12.0</v>
       </c>
-      <c r="H33" s="6">
+      <c r="H33" s="7">
         <v>339039.0</v>
       </c>
-      <c r="I33" s="6">
+      <c r="I33" s="7">
         <v>2048.0</v>
       </c>
-      <c r="J33" s="10">
+      <c r="J33" s="13">
         <v>173846.38</v>
       </c>
-      <c r="K33" s="6">
+      <c r="K33" s="7">
         <v>0.0</v>
       </c>
-      <c r="L33" s="10">
+      <c r="L33" s="13">
         <v>173846.38</v>
       </c>
       <c r="AB33" s="2"/>
@@ -9492,40 +9492,40 @@
       <c r="AH33" s="2"/>
     </row>
     <row r="34">
-      <c r="A34" s="6" t="s">
+      <c r="A34" s="7" t="s">
         <v>134</v>
       </c>
-      <c r="B34" s="6" t="s">
+      <c r="B34" s="7" t="s">
         <v>135</v>
       </c>
-      <c r="C34" s="6" t="s">
-        <v>136</v>
-      </c>
-      <c r="D34" s="6" t="s">
-        <v>3</v>
-      </c>
-      <c r="E34" s="9">
+      <c r="C34" s="7" t="s">
+        <v>137</v>
+      </c>
+      <c r="D34" s="7" t="s">
+        <v>4</v>
+      </c>
+      <c r="E34" s="10">
         <v>46240.0</v>
       </c>
-      <c r="F34" s="6" t="s">
-        <v>4</v>
-      </c>
-      <c r="G34" s="6">
+      <c r="F34" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="G34" s="7">
         <v>12.0</v>
       </c>
-      <c r="H34" s="6">
+      <c r="H34" s="7">
         <v>339039.0</v>
       </c>
-      <c r="I34" s="6" t="s">
-        <v>137</v>
-      </c>
-      <c r="J34" s="10">
+      <c r="I34" s="7" t="s">
+        <v>140</v>
+      </c>
+      <c r="J34" s="13">
         <v>236343.68</v>
       </c>
-      <c r="K34" s="6">
+      <c r="K34" s="7">
         <v>0.0</v>
       </c>
-      <c r="L34" s="10">
+      <c r="L34" s="13">
         <v>236343.68</v>
       </c>
       <c r="AB34" s="2"/>
@@ -9537,40 +9537,40 @@
       <c r="AH34" s="2"/>
     </row>
     <row r="35">
-      <c r="A35" s="6" t="s">
-        <v>138</v>
-      </c>
-      <c r="B35" s="6" t="s">
+      <c r="A35" s="7" t="s">
+        <v>141</v>
+      </c>
+      <c r="B35" s="7" t="s">
         <v>125</v>
       </c>
-      <c r="C35" s="6" t="s">
-        <v>139</v>
-      </c>
-      <c r="D35" s="6" t="s">
-        <v>3</v>
-      </c>
-      <c r="E35" s="9">
+      <c r="C35" s="7" t="s">
+        <v>143</v>
+      </c>
+      <c r="D35" s="7" t="s">
+        <v>4</v>
+      </c>
+      <c r="E35" s="10">
         <v>46282.0</v>
       </c>
-      <c r="F35" s="6" t="s">
-        <v>4</v>
-      </c>
-      <c r="G35" s="6">
+      <c r="F35" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="G35" s="7">
         <v>12.0</v>
       </c>
-      <c r="H35" s="6">
+      <c r="H35" s="7">
         <v>339039.0</v>
       </c>
-      <c r="I35" s="6" t="s">
+      <c r="I35" s="7" t="s">
         <v>104</v>
       </c>
-      <c r="J35" s="10">
+      <c r="J35" s="13">
         <v>1145462.93</v>
       </c>
-      <c r="K35" s="6">
+      <c r="K35" s="7">
         <v>0.0</v>
       </c>
-      <c r="L35" s="10">
+      <c r="L35" s="13">
         <v>1145462.93</v>
       </c>
       <c r="AB35" s="2"/>

</xml_diff>